<commit_message>
docs(w39): tracker -- MON-03 notify audit, EX-20 SIP fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DARnfJBdfCsR1TUSafW4VA
</commit_message>
<xml_diff>
--- a/docs/ATIP_Master_Deployment_Tracker_Wave_1_to_20_UPDATED.xlsx
+++ b/docs/ATIP_Master_Deployment_Tracker_Wave_1_to_20_UPDATED.xlsx
@@ -11248,12 +11248,12 @@
       </c>
       <c r="V66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>W1 developed 2026-09-24 — not yet independently validated (docs/W1_FOUNDATION_HANDOFF.md)</t>
+          <t>W1 developed 2026-09-24 — not yet independently validated (docs/W1_FOUNDATION_HANDOFF.md) | W39 audit of every notify path: an alert sent while the caller held an uncommitted write stalled 60 s and was lost -- fixed in SIP run_due, the wealth investor cycle, the Dhan live-quote refresh and portfolio sync; log_job and the Dhan tick / index flushes now close on failure (tests/test_w39_notify_transactions.py)</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
@@ -39331,7 +39331,7 @@
       </c>
       <c r="Q308" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_retail.py</t>
+          <t>tests/test_w39_retail.py; tests/test_w39_notify_transactions.py</t>
         </is>
       </c>
       <c r="R308" s="2" t="inlineStr">
@@ -39353,7 +39353,7 @@
       </c>
       <c r="W308" s="2" t="inlineStr">
         <is>
-          <t>W39 developed 2026-10-07 on branch claude/wizardly-curie-fbjeoa (PR #5); independent validation PENDING</t>
+          <t>W39 developed 2026-10-07 (PR #5); fix: with two or more plans due, the second order waited on the first plan's uncommitted rows and failed -- the loop now commits before each placement</t>
         </is>
       </c>
       <c r="X308" s="2" t="inlineStr">
@@ -39363,7 +39363,7 @@
       </c>
       <c r="Y308" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_retail.py | 87% of 149 lines in 1 key file(s) run by: test_w39_retail, test_w39_ui_smoke</t>
+          <t>tests/test_w39_retail.py; tests/test_w39_notify_transactions.py | 87% of 149 lines in 1 key file(s) run by: test_w39_retail, test_w39_ui_smoke</t>
         </is>
       </c>
       <c r="Z308" s="2" t="inlineStr"/>
@@ -43102,7 +43102,7 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_retail.py</t>
+          <t>tests/test_w39_retail.py; tests/test_w39_notify_transactions.py</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
@@ -43124,7 +43124,7 @@
       </c>
       <c r="W31" s="2" t="inlineStr">
         <is>
-          <t>W39 developed 2026-10-07 on branch claude/wizardly-curie-fbjeoa (PR #5); independent validation PENDING</t>
+          <t>W39 developed 2026-10-07 (PR #5); fix: with two or more plans due, the second order waited on the first plan's uncommitted rows and failed -- the loop now commits before each placement</t>
         </is>
       </c>
       <c r="X31" s="2" t="inlineStr">
@@ -43134,7 +43134,7 @@
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_retail.py | 87% of 149 lines in 1 key file(s) run by: test_w39_retail, test_w39_ui_smoke</t>
+          <t>tests/test_w39_retail.py; tests/test_w39_notify_transactions.py | 87% of 149 lines in 1 key file(s) run by: test_w39_retail, test_w39_ui_smoke</t>
         </is>
       </c>
       <c r="Z31" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(w40): tracker regenerated -- 333 rows, coverage from 1,556 passing tests
126 COMPLETED, 197 IMPLEMENTED BUT NOT VERIFIED, 9 BLOCKED, 1 IN PROGRESS;
W40-RISKMODEL and W40-META added, eleven rows updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DARnfJBdfCsR1TUSafW4VA
</commit_message>
<xml_diff>
--- a/docs/ATIP_Master_Deployment_Tracker_Wave_1_to_20_UPDATED.xlsx
+++ b/docs/ATIP_Master_Deployment_Tracker_Wave_1_to_20_UPDATED.xlsx
@@ -22,8 +22,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Legend" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Features'!$A$1:$Z$332</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Items (W39)'!$A$1:$Z$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Features'!$A$1:$Z$334</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Items (W39)'!$A$1:$Z$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Blockers'!$A$1:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Master Tracker'!$A$1:$H$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Gap Analysis'!$A$1:$E$15</definedName>
@@ -32,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'PERF-001 Detail'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Implementation Sequence'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Master Dev Prompt'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Owner CSV vs repo'!$A$1:$G$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Owner CSV vs repo'!$A$1:$G$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>207</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14">
@@ -787,7 +787,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23">
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -825,7 +825,7 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25">
@@ -1132,55 +1132,58 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>W40 (PR #9)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Features</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Developed</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>0 Delivered baseline (maintain)</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>58</v>
-      </c>
-      <c r="C43" t="n">
-        <v>58</v>
-      </c>
-      <c r="D43" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1 Foundation</t>
+          <t>0 Delivered baseline (maintain)</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="C44" t="n">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1189,14 +1192,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2 Quant Research (data, factors, backtesting)</t>
+          <t>1 Foundation</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="C45" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1205,14 +1208,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>3 Strategy Engine</t>
+          <t>2 Quant Research (data, factors, backtesting)</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="C46" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
@@ -1221,78 +1224,78 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>4 AI/ML</t>
+          <t>3 Strategy Engine</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C47" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5 Risk &amp; Portfolio</t>
+          <t>4 AI/ML</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>6 Execution</t>
+          <t>5 Risk &amp; Portfolio</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C49" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>7 Advanced Quant</t>
+          <t>6 Execution</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C50" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>8 Production Hardening</t>
+          <t>7 Advanced Quant</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -1301,14 +1304,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>8 Production hardening</t>
+          <t>8 Production Hardening</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C52" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -1317,48 +1320,64 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>9 Enterprise SaaS (final objective)</t>
+          <t>8 Production hardening</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C53" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>10 Wealth track (Waves 11-20)</t>
+          <t>9 Enterprise SaaS (final objective)</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="C54" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>10 Wealth track (Waves 11-20)</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>11</v>
+      </c>
+      <c r="C55" t="n">
+        <v>9</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>11 W39 reconciliation (owner tracker 2026-10-07)</t>
         </is>
       </c>
-      <c r="B55" t="n">
-        <v>54</v>
-      </c>
-      <c r="C55" t="n">
-        <v>53</v>
-      </c>
-      <c r="D55" t="n">
+      <c r="B56" t="n">
+        <v>56</v>
+      </c>
+      <c r="C56" t="n">
+        <v>55</v>
+      </c>
+      <c r="D56" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2544,7 +2563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2596,12 +2615,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BT-14</t>
+          <t>BT-04</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Robustness</t>
+          <t>Parameter optimisation</t>
         </is>
       </c>
       <c r="C2" s="18" t="inlineStr">
@@ -2626,29 +2645,29 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>W23: robustness battery (costs x2, slippage x3, universe halves, period halves, regimes, Monte Carlo) with verdict. W39b: backtest/cpcv.py -- combinatorial purg</t>
+          <t>W23: grid / random / adaptive optimiser with trial runs, test-window refusal, Deflated Sharpe + overfit warning. W40: method="bayes" -- a Tree-structured Parzen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DP-08</t>
+          <t>BT-14</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Derivatives data</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+          <t>Robustness</t>
+        </is>
+      </c>
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E3" s="18" t="inlineStr">
@@ -2658,24 +2677,24 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>90</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
+          <t>W23: robustness battery (costs x2, slippage x3, universe halves, period halves, regimes, Monte Carlo) with verdict. W39b: backtest/cpcv.py -- combinatorial purg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SE-05</t>
+          <t>DP-08</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AI-driven strategies</t>
+          <t>Derivatives data</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -2685,71 +2704,71 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>W5 developed 2026-09-25 (incl. completion pass) — framework only, no model trained or validated; independent testing PENDING (ChatGPT); see docs/W5_AI_ML_HANDOF</t>
+          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NS-05</t>
+          <t>SE-05</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Novelty/decay/source weighting</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
+          <t>AI-driven strategies</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>W28b developed 2026-10-01 on branch w28b-news-weighting (on w33-wealth-qa) — independent validation PENDING (ChatGPT); see docs/W28B_NEWS_WEIGHTING_HANDOFF.md |</t>
+          <t>W5 developed 2026-09-25 (incl. completion pass) — framework only, no model trained or validated; independent testing PENDING (ChatGPT); see docs/W5_AI_ML_HANDOF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NS-06</t>
+          <t>NS-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Earnings call / announcement NLP</t>
+          <t>Novelty/decay/source weighting</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
@@ -2759,7 +2778,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -2769,7 +2788,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2781,12 +2800,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ML-02</t>
+          <t>NS-06</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Deep learning</t>
+          <t>Earnings call / announcement NLP</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
@@ -2806,24 +2825,24 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
+          <t>W28b developed 2026-10-01 on branch w28b-news-weighting (on w33-wealth-qa) — independent validation PENDING (ChatGPT); see docs/W28B_NEWS_WEIGHTING_HANDOFF.md |</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ML-04</t>
+          <t>ML-02</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Reinforcement learning</t>
+          <t>Deep learning</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
@@ -2843,7 +2862,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2855,59 +2874,59 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PF-06</t>
+          <t>ML-04</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Rebalancing</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
+          <t>Reinforcement learning</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>W6 developed 2026-09-25 — coding only; independent testing PENDING (ChatGPT); see docs/W6_ADVANCED_QUANT_HANDOFF.md</t>
+          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>DP-04</t>
+          <t>PF-06</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Tick data</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
+          <t>Rebalancing</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
@@ -2917,24 +2936,24 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>90</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
+          <t>W6 developed 2026-09-25 — coding only; independent testing PENDING (ChatGPT); see docs/W6_ADVANCED_QUANT_HANDOFF.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DP-05</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Order book / depth</t>
+          <t>Tick data</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
@@ -2966,22 +2985,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AF-06</t>
+          <t>DP-05</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Derivatives factors</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>Order book / depth</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
@@ -2991,34 +3010,34 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
+          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EX-11</t>
+          <t>AF-06</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Execution algos</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
+          <t>Derivatives factors</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
@@ -3033,29 +3052,29 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>W34 developed 2026-10-01 on branch w34-execution-microstructure — independent validation PENDING (ChatGPT); see docs/W34_EXECUTION_MICROSTRUCTURE_HANDOFF.md | W</t>
+          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>EX-12</t>
+          <t>QR-05</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Market impact model</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
+          <t>Stat-arb / pairs / cointegration</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>85</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
@@ -3065,24 +3084,24 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>W34 developed 2026-10-01 on branch w34-execution-microstructure — independent validation PENDING (ChatGPT); see docs/W34_EXECUTION_MICROSTRUCTURE_HANDOFF.md | W</t>
+          <t>W6 developed 2026-09-25 — coding only; independent testing PENDING (ChatGPT); see docs/W6_ADVANCED_QUANT_HANDOFF.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>EX-15</t>
+          <t>EX-11</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Latency telemetry</t>
+          <t>Execution algos</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
@@ -3114,12 +3133,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>EX-16</t>
+          <t>EX-12</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Event-driven OMS</t>
+          <t>Market impact model</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
@@ -3129,7 +3148,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -3151,12 +3170,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BT-17</t>
+          <t>EX-15</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Event-driven backtester</t>
+          <t>Latency telemetry</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
@@ -3188,12 +3207,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DP-14</t>
+          <t>EX-16</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Macroeconomic data</t>
+          <t>Event-driven OMS</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
@@ -3203,7 +3222,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -3218,19 +3237,19 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
+          <t>W34 developed 2026-10-01 on branch w34-execution-microstructure — independent validation PENDING (ChatGPT); see docs/W34_EXECUTION_MICROSTRUCTURE_HANDOFF.md | W</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AD-01</t>
+          <t>BT-17</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Alt-data framework</t>
+          <t>Event-driven backtester</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
@@ -3255,19 +3274,19 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
+          <t>W34 developed 2026-10-01 on branch w34-execution-microstructure — independent validation PENDING (ChatGPT); see docs/W34_EXECUTION_MICROSTRUCTURE_HANDOFF.md | W</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AD-02</t>
+          <t>DP-14</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Alt-data sources</t>
+          <t>Macroeconomic data</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
@@ -3287,7 +3306,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -3299,12 +3318,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DP-22</t>
+          <t>AD-01</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Point-in-time data lake</t>
+          <t>Alt-data framework</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -3314,7 +3333,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -3336,12 +3355,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DP-21</t>
+          <t>AD-02</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Multi-asset data</t>
+          <t>Alt-data sources</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
@@ -3366,56 +3385,56 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check: AMFI mutual-</t>
+          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>API-05</t>
+          <t>DP-22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>API contracts/docs</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
+          <t>Point-in-time data lake</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
-        </is>
-      </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>W8 developed 2026-09-25 (production hardening) — coding only; independent testing PENDING (ChatGPT); see docs/W8_PRODUCTION_HARDENING_HANDOFF.md</t>
+          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check 2026-10-07: c</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>API-06</t>
+          <t>DP-21</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Widget JSON schemas</t>
+          <t>Multi-asset data</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
@@ -3425,7 +3444,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
@@ -3435,34 +3454,34 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>70</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
+          <t>W35 developed 2026-10-01 on branch w35-data-platform — independent validation PENDING (ChatGPT); see docs/W35_DATA_PLATFORM_HANDOFF.md | W39 check: AMFI mutual-</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>DBS-05</t>
+          <t>API-05</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Scalable database</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
+          <t>API contracts/docs</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>95</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -3472,24 +3491,24 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>W38 developed 2026-10-02 on branch w38-platform-compliance; 15 new tests + full suite pass; independent validation PENDING (ChatGPT); see docs/W38_PLATFORM_COMP</t>
+          <t>W8 developed 2026-09-25 (production hardening) — coding only; independent testing PENDING (ChatGPT); see docs/W8_PRODUCTION_HARDENING_HANDOFF.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ENT-06</t>
+          <t>API-06</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Per-user broker credential vault</t>
+          <t>Widget JSON schemas</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
@@ -3499,7 +3518,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E26" s="18" t="inlineStr">
@@ -3514,19 +3533,19 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>W37 developed 2026-10-02 on branch w37-brokers-multi-asset; 9 new tests + full suite 508/508 pass; independent validation PENDING (ChatGPT); see docs/W37_BROKER</t>
+          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ENT-14</t>
+          <t>DBS-05</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Regulatory approvals</t>
+          <t>Scalable database</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
@@ -3539,14 +3558,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E27" s="19" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>70</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3558,12 +3577,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SEC-05</t>
+          <t>ENT-06</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Compliance monitoring</t>
+          <t>Per-user broker credential vault</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
@@ -3583,24 +3602,24 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>W38 developed 2026-10-02 on branch w38-platform-compliance; 15 new tests + full suite pass; independent validation PENDING (ChatGPT); see docs/W38_PLATFORM_COMP</t>
+          <t>W37 developed 2026-10-02 on branch w37-brokers-multi-asset; 9 new tests + full suite 508/508 pass; independent validation PENDING (ChatGPT); see docs/W37_BROKER</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ENT-17</t>
+          <t>ENT-14</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Data privacy</t>
+          <t>Regulatory approvals</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
@@ -3613,14 +3632,14 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E29" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3632,49 +3651,49 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ENT-04</t>
+          <t>SEC-05</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Subscriptions &amp; billing</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+          <t>Compliance monitoring</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>W7 developed 2026-09-25 (enterprise layer, off by default) — coding only; independent testing PENDING (ChatGPT); see docs/W7_ENTERPRISE_HANDOFF.md</t>
+          <t>W38 developed 2026-10-02 on branch w38-platform-compliance; 15 new tests + full suite pass; independent validation PENDING (ChatGPT); see docs/W38_PLATFORM_COMP</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ENT-09</t>
+          <t>ENT-17</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Mobile apps</t>
+          <t>Data privacy</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
@@ -3694,7 +3713,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -3706,27 +3725,27 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>API-03</t>
+          <t>ENT-04</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Versioned public API</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+          <t>Subscriptions &amp; billing</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="E32" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3736,19 +3755,19 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>W8 developed 2026-09-25 (production hardening) — coding only; independent testing PENDING (ChatGPT); see docs/W8_PRODUCTION_HARDENING_HANDOFF.md</t>
+          <t>W7 developed 2026-09-25 (enterprise layer, off by default) — coding only; independent testing PENDING (ChatGPT); see docs/W7_ENTERPRISE_HANDOFF.md</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PF-12</t>
+          <t>ENT-09</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Multi-broker import</t>
+          <t>Mobile apps</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
@@ -3768,34 +3787,34 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>W37 developed 2026-10-02 on branch w37-brokers-multi-asset; 9 new tests + full suite 508/508 pass; independent validation PENDING (ChatGPT); see docs/W37_BROKER</t>
+          <t>W38 developed 2026-10-02 on branch w38-platform-compliance; 15 new tests + full suite pass; independent validation PENDING (ChatGPT); see docs/W38_PLATFORM_COMP</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BR-07</t>
+          <t>API-03</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Additional brokers</t>
-        </is>
-      </c>
-      <c r="C34" s="17" t="inlineStr">
-        <is>
-          <t>YET TO START</t>
+          <t>Versioned public API</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
@@ -3805,24 +3824,24 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>90</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>W37 developed 2026-10-02 on branch w37-brokers-multi-asset; 9 new tests + full suite 508/508 pass; independent validation PENDING (ChatGPT); see docs/W37_BROKER</t>
+          <t>W8 developed 2026-09-25 (production hardening) — coding only; independent testing PENDING (ChatGPT); see docs/W8_PRODUCTION_HARDENING_HANDOFF.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ENT-15</t>
+          <t>PF-12</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Multi-asset trading</t>
+          <t>Multi-broker import</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
@@ -3842,7 +3861,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -3854,12 +3873,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SE-10</t>
+          <t>BR-07</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>No/low-code strategy builder</t>
+          <t>Additional brokers</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
@@ -3879,24 +3898,24 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
+          <t>W37 developed 2026-10-02 on branch w37-brokers-multi-asset; 9 new tests + full suite 508/508 pass; independent validation PENDING (ChatGPT); see docs/W37_BROKER</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ML-16</t>
+          <t>ENT-15</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>AI chat assistant</t>
+          <t>Multi-asset trading</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
@@ -3921,19 +3940,19 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
+          <t>W37 developed 2026-10-02 on branch w37-brokers-multi-asset; 9 new tests + full suite 508/508 pass; independent validation PENDING (ChatGPT); see docs/W37_BROKER</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>OPS-04</t>
+          <t>SE-10</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Cloud deployment</t>
+          <t>No/low-code strategy builder</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
@@ -3953,98 +3972,98 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>W38 developed 2026-10-02 on branch w38-platform-compliance; 15 new tests + full suite pass; independent validation PENDING (ChatGPT); see docs/W38_PLATFORM_COMP</t>
+          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ENT-16</t>
+          <t>ML-16</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Scalability, HA &amp; observability</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+          <t>AI chat assistant</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>W8 developed 2026-09-25 (production hardening) — coding only; independent testing PENDING (ChatGPT); see docs/W8_PRODUCTION_HARDENING_HANDOFF.md</t>
+          <t>W36 developed 2026-10-02 on branch w36-ml-strategy-tooling; 13 new tests + full suite 499/499 pass; independent validation PENDING (ChatGPT); see docs/W36_ML_ST</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>PERF-001</t>
+          <t>OPS-04</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Investor performance attribution</t>
-        </is>
-      </c>
-      <c r="C40" s="18" t="inlineStr">
+          <t>Cloud deployment</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>YET TO START</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
         <is>
           <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="E40" s="18" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED BUT NOT VERIFIED</t>
-        </is>
-      </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>branch w20-release; merged to master; not deployed | W39 check 2026-10-07: commit is an ancestor of master</t>
+          <t>W38 developed 2026-10-02 on branch w38-platform-compliance; 15 new tests + full suite pass; independent validation PENDING (ChatGPT); see docs/W38_PLATFORM_COMP</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>QA-001</t>
+          <t>ENT-16</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Wealth QA / security / performance</t>
+          <t>Scalability, HA &amp; observability</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
@@ -4054,64 +4073,138 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>50</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>RC line = w33-wealth-qa (W11-W32); merged to master; not deployed | W39 check 2026-10-07: commit is an ancestor of master</t>
+          <t>W8 developed 2026-09-25 (production hardening) — coding only; independent testing PENDING (ChatGPT); see docs/W8_PRODUCTION_HARDENING_HANDOFF.md</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>PERF-001</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Investor performance attribution</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>branch w20-release; merged to master; not deployed | W39 check 2026-10-07: commit is an ancestor of master</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>QA-001</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Wealth QA / security / performance</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>RC line = w33-wealth-qa (W11-W32); merged to master; not deployed | W39 check 2026-10-07: commit is an ancestor of master</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>UAT-001</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Beta / UAT</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C44" s="15" t="inlineStr">
         <is>
           <t>IN PROGRESS</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
+      <c r="E44" s="19" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>RC line = w33-wealth-qa; merged to master; not deployed | W39 check 2026-10-07: commit is an ancestor of master</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G42"/>
+  <autoFilter ref="A1:G44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4284,7 +4377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z332"/>
+  <dimension ref="A1:Z334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4754,7 +4847,7 @@
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>92% of 24 lines in 1 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_regressions, test_risk_controls (+21 more)</t>
+          <t>95% of 41 lines in 1 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_regressions, test_risk_controls (+28 more)</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr"/>
@@ -4858,7 +4951,7 @@
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib</t>
+          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr"/>
@@ -4962,7 +5055,7 @@
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib</t>
+          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr"/>
@@ -5066,7 +5159,7 @@
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_technical_rs_fib.py | 86% of 728 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w39_untested_modules</t>
+          <t>tests/test_w39_technical_rs_fib.py | 86% of 728 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w39_untested_modules, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr"/>
@@ -5170,7 +5263,7 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib</t>
+          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr"/>
@@ -6106,7 +6199,7 @@
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>86% of 346 lines in 1 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>86% of 346 lines in 1 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z17" s="2" t="inlineStr"/>
@@ -6210,7 +6303,7 @@
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>35% of 1222 lines in 1 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+1 more)</t>
+          <t>35% of 1229 lines in 1 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+2 more)</t>
         </is>
       </c>
       <c r="Z18" s="2" t="inlineStr"/>
@@ -6522,7 +6615,7 @@
       </c>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>64% of 300 lines in 1 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_exec_data_tests, test_w39_notify_transactions, test_w39_perf_budget, test_w39_performance_detail (+5 more)</t>
+          <t>64% of 301 lines in 1 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_exec_data_tests, test_w39_notify_transactions, test_w39_perf_budget, test_w39_performance_detail (+6 more)</t>
         </is>
       </c>
       <c r="Z21" s="2" t="inlineStr"/>
@@ -6626,7 +6719,7 @@
       </c>
       <c r="Y22" s="2" t="inlineStr">
         <is>
-          <t>64% of 300 lines in 1 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_exec_data_tests, test_w39_notify_transactions, test_w39_perf_budget, test_w39_performance_detail (+5 more)</t>
+          <t>64% of 301 lines in 1 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_exec_data_tests, test_w39_notify_transactions, test_w39_perf_budget, test_w39_performance_detail (+6 more)</t>
         </is>
       </c>
       <c r="Z22" s="2" t="inlineStr"/>
@@ -6938,7 +7031,7 @@
       </c>
       <c r="Y25" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z25" s="2" t="inlineStr"/>
@@ -7042,7 +7135,7 @@
       </c>
       <c r="Y26" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z26" s="2" t="inlineStr"/>
@@ -7146,7 +7239,7 @@
       </c>
       <c r="Y27" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z27" s="2" t="inlineStr"/>
@@ -7250,7 +7343,7 @@
       </c>
       <c r="Y28" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z28" s="2" t="inlineStr"/>
@@ -7978,7 +8071,7 @@
       </c>
       <c r="Y35" s="2" t="inlineStr">
         <is>
-          <t>tests/test_paper_broker.py | 55% of 321 lines in 1 key file(s) run by: test_paper_broker, test_risk_controls, test_strategy_live, test_w37_brokers_multi_asset, test_w39_exec_data_tests, test_w39_performance_detail, test_w39_qa_suite, test_wealth_dna_holdings (+1 more)</t>
+          <t>tests/test_paper_broker.py | 55% of 321 lines in 1 key file(s) run by: test_paper_broker, test_risk_controls, test_strategy_live, test_w37_brokers_multi_asset, test_w39_exec_data_tests, test_w39_performance_detail, test_w39_qa_suite, test_w40_futures_backtest (+4 more)</t>
         </is>
       </c>
       <c r="Z35" s="2" t="inlineStr"/>
@@ -8394,7 +8487,7 @@
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z39" s="2" t="inlineStr"/>
@@ -8498,7 +8591,7 @@
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z40" s="2" t="inlineStr"/>
@@ -8602,7 +8695,7 @@
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr"/>
@@ -8706,7 +8799,7 @@
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z42" s="2" t="inlineStr"/>
@@ -8810,7 +8903,7 @@
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z43" s="2" t="inlineStr"/>
@@ -8914,7 +9007,7 @@
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z44" s="2" t="inlineStr"/>
@@ -9018,7 +9111,7 @@
       </c>
       <c r="Y45" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z45" s="2" t="inlineStr"/>
@@ -9122,7 +9215,7 @@
       </c>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z46" s="2" t="inlineStr"/>
@@ -9226,7 +9319,7 @@
       </c>
       <c r="Y47" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z47" s="2" t="inlineStr"/>
@@ -9330,7 +9423,7 @@
       </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z48" s="2" t="inlineStr"/>
@@ -9434,7 +9527,7 @@
       </c>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z49" s="2" t="inlineStr"/>
@@ -9642,7 +9735,7 @@
       </c>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>65% of 808 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+29 more)</t>
+          <t>64% of 812 lines in 1 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+36 more)</t>
         </is>
       </c>
       <c r="Z51" s="2" t="inlineStr"/>
@@ -9746,7 +9839,7 @@
       </c>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>93% of 43 lines in 1 key file(s) run by: test_auto_recover, test_risk_controls, test_w38_platform_compliance, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+24 more)</t>
+          <t>93% of 43 lines in 1 key file(s) run by: test_auto_recover, test_risk_controls, test_w38_platform_compliance, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+30 more)</t>
         </is>
       </c>
       <c r="Z52" s="2" t="inlineStr"/>
@@ -9850,7 +9943,7 @@
       </c>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>86% of 346 lines in 1 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>86% of 346 lines in 1 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z53" s="2" t="inlineStr"/>
@@ -10178,7 +10271,7 @@
       </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>78% of 234 lines in 1 key file(s) run by: test_fii_dii_and_delivery_factor, test_index_feed, test_risk_controls, test_w39_notify_transactions</t>
+          <t>76% of 234 lines in 1 key file(s) run by: test_fii_dii_and_delivery_factor, test_index_feed, test_regressions, test_w39_notify_transactions</t>
         </is>
       </c>
       <c r="Z56" s="2" t="inlineStr"/>
@@ -10298,7 +10391,7 @@
       </c>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>69% of 360 lines in 2 key file(s) run by: test_auto_recover, test_w39_ops_tests, test_w39_perf_budget, test_w39b_razorpay</t>
+          <t>68% of 360 lines in 2 key file(s) run by: test_auto_recover, test_w39_ops_tests, test_w39_perf_budget, test_w39b_razorpay</t>
         </is>
       </c>
       <c r="Z57" s="2" t="inlineStr"/>
@@ -10622,7 +10715,7 @@
       </c>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>47% of 3163 lines in 5 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_job_monitoring, test_market_health, test_regressions, test_risk_controls, test_signal_pipeline (+8 more)</t>
+          <t>46% of 3170 lines in 5 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_job_monitoring, test_market_health, test_regressions, test_risk_controls, test_signal_pipeline (+9 more)</t>
         </is>
       </c>
       <c r="Z60" s="2" t="inlineStr"/>
@@ -10742,7 +10835,7 @@
       </c>
       <c r="Y61" s="2" t="inlineStr">
         <is>
-          <t>85% of 936 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>85% of 936 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z61" s="2" t="inlineStr"/>
@@ -10862,7 +10955,7 @@
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>47% of 3163 lines in 5 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_job_monitoring, test_market_health, test_regressions, test_risk_controls, test_signal_pipeline (+8 more)</t>
+          <t>46% of 3170 lines in 5 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_job_monitoring, test_market_health, test_regressions, test_risk_controls, test_signal_pipeline (+9 more)</t>
         </is>
       </c>
       <c r="Z62" s="2" t="inlineStr"/>
@@ -10982,7 +11075,7 @@
       </c>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>72% of 1105 lines in 3 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>72% of 1105 lines in 3 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z63" s="2" t="inlineStr"/>
@@ -11098,7 +11191,7 @@
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>46% of 1568 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>46% of 1575 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z64" s="2" t="inlineStr"/>
@@ -11218,7 +11311,7 @@
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>39% of 1338 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_risk_controls, test_signal_pipeline, test_w38_platform_compliance, test_w39_api_contract, test_w39_exec_data_tests (+7 more)</t>
+          <t>39% of 1345 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_risk_controls, test_signal_pipeline, test_w38_platform_compliance, test_w39_api_contract, test_w39_exec_data_tests (+8 more)</t>
         </is>
       </c>
       <c r="Z65" s="2" t="inlineStr"/>
@@ -11338,7 +11431,7 @@
       </c>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>64% of 1070 lines in 2 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_api_contract, test_w39_backtest (+31 more)</t>
+          <t>63% of 1074 lines in 2 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_api_contract, test_w39_backtest (+38 more)</t>
         </is>
       </c>
       <c r="Z66" s="2" t="inlineStr"/>
@@ -11578,7 +11671,7 @@
       </c>
       <c r="Y68" s="2" t="inlineStr">
         <is>
-          <t>66% of 502 lines in 2 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 502 lines in 2 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z68" s="2" t="inlineStr"/>
@@ -11810,7 +11903,7 @@
       </c>
       <c r="Y70" s="2" t="inlineStr">
         <is>
-          <t>57% of 515 lines in 3 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>57% of 515 lines in 3 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z70" s="2" t="inlineStr"/>
@@ -11930,7 +12023,7 @@
       </c>
       <c r="Y71" s="2" t="inlineStr">
         <is>
-          <t>31% of 1391 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+1 more)</t>
+          <t>31% of 1398 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+2 more)</t>
         </is>
       </c>
       <c r="Z71" s="2" t="inlineStr"/>
@@ -12266,7 +12359,7 @@
       </c>
       <c r="Y74" s="2" t="inlineStr">
         <is>
-          <t>test_postmarket_scores_a_seeded_session_end_to_end; test_postmarket_refuses_a_session_that_is_a_copy_of_the_previous_one | 35% of 1222 lines in 1 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+1 more)</t>
+          <t>test_postmarket_scores_a_seeded_session_end_to_end; test_postmarket_refuses_a_session_that_is_a_copy_of_the_previous_one | 35% of 1229 lines in 1 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+2 more)</t>
         </is>
       </c>
       <c r="Z74" s="2" t="inlineStr"/>
@@ -12378,7 +12471,7 @@
       </c>
       <c r="Y75" s="2" t="inlineStr">
         <is>
-          <t>30% of 1676 lines in 4 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_fundamentals_screener, test_job_monitoring, test_signal_pipeline, test_w38_platform_compliance, test_w39_history, test_w39_notify_transactions (+3 more)</t>
+          <t>30% of 1683 lines in 4 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_fundamentals_screener, test_job_monitoring, test_signal_pipeline, test_w38_platform_compliance, test_w39_history, test_w39_notify_transactions (+4 more)</t>
         </is>
       </c>
       <c r="Z75" s="2" t="inlineStr"/>
@@ -12942,7 +13035,7 @@
       </c>
       <c r="Y80" s="2" t="inlineStr">
         <is>
-          <t>41% of 881 lines in 2 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_risk_gateway (+2 more)</t>
+          <t>40% of 881 lines in 2 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_risk_gateway (+2 more)</t>
         </is>
       </c>
       <c r="Z80" s="2" t="inlineStr"/>
@@ -13062,7 +13155,7 @@
       </c>
       <c r="Y81" s="2" t="inlineStr">
         <is>
-          <t>39% of 1338 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_risk_controls, test_signal_pipeline, test_w38_platform_compliance, test_w39_api_contract, test_w39_exec_data_tests (+7 more)</t>
+          <t>39% of 1345 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_risk_controls, test_signal_pipeline, test_w38_platform_compliance, test_w39_api_contract, test_w39_exec_data_tests (+8 more)</t>
         </is>
       </c>
       <c r="Z81" s="2" t="inlineStr"/>
@@ -13182,7 +13275,7 @@
       </c>
       <c r="Y82" s="2" t="inlineStr">
         <is>
-          <t>63% of 942 lines in 2 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+33 more)</t>
+          <t>62% of 946 lines in 2 key file(s) run by: test_auto_recover, test_index_feed, test_job_monitoring, test_regressions, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20 (+40 more)</t>
         </is>
       </c>
       <c r="Z82" s="2" t="inlineStr"/>
@@ -13302,7 +13395,7 @@
       </c>
       <c r="Y83" s="2" t="inlineStr">
         <is>
-          <t>76% of 480 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>76% of 480 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z83" s="2" t="inlineStr"/>
@@ -13418,7 +13511,7 @@
       </c>
       <c r="Y84" s="2" t="inlineStr">
         <is>
-          <t>70% of 807 lines in 2 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_exec_data_tests (+8 more)</t>
+          <t>70% of 807 lines in 2 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_exec_data_tests (+13 more)</t>
         </is>
       </c>
       <c r="Z84" s="2" t="inlineStr"/>
@@ -13538,7 +13631,7 @@
       </c>
       <c r="Y85" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z85" s="2" t="inlineStr"/>
@@ -13658,7 +13751,7 @@
       </c>
       <c r="Y86" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z86" s="2" t="inlineStr"/>
@@ -14110,7 +14203,7 @@
       </c>
       <c r="Y90" s="2" t="inlineStr">
         <is>
-          <t>40% of 1345 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+1 more)</t>
+          <t>40% of 1352 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+2 more)</t>
         </is>
       </c>
       <c r="Z90" s="2" t="inlineStr"/>
@@ -14230,7 +14323,7 @@
       </c>
       <c r="Y91" s="2" t="inlineStr">
         <is>
-          <t>83% of 459 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>83% of 459 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z91" s="2" t="inlineStr"/>
@@ -14454,7 +14547,7 @@
       </c>
       <c r="Y93" s="2" t="inlineStr">
         <is>
-          <t>58% of 1170 lines in 3 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>58% of 1170 lines in 3 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z93" s="2" t="inlineStr"/>
@@ -14566,7 +14659,7 @@
       </c>
       <c r="Y94" s="2" t="inlineStr">
         <is>
-          <t>86% of 728 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w39_untested_modules</t>
+          <t>86% of 728 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w39_untested_modules, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z94" s="2" t="inlineStr"/>
@@ -14674,7 +14767,7 @@
       </c>
       <c r="Y95" s="2" t="inlineStr">
         <is>
-          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib</t>
+          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z95" s="2" t="inlineStr"/>
@@ -15006,7 +15099,7 @@
       </c>
       <c r="Y98" s="2" t="inlineStr">
         <is>
-          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib</t>
+          <t>80% of 357 lines in 1 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z98" s="2" t="inlineStr"/>
@@ -15230,7 +15323,7 @@
       </c>
       <c r="Y100" s="2" t="inlineStr">
         <is>
-          <t>61% of 266 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio</t>
+          <t>68% of 269 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z100" s="2" t="inlineStr"/>
@@ -15454,7 +15547,7 @@
       </c>
       <c r="Y102" s="2" t="inlineStr">
         <is>
-          <t>61% of 266 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio</t>
+          <t>68% of 269 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z102" s="2" t="inlineStr"/>
@@ -16094,9 +16187,9 @@
           <t>COMPLETED</t>
         </is>
       </c>
-      <c r="K108" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="K108" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="L108" s="2" t="inlineStr">
@@ -16162,7 +16255,7 @@
       </c>
       <c r="Y108" s="2" t="inlineStr">
         <is>
-          <t>46% of 242 lines in 3 key file(s) run by: test_auto_recover, test_w39_quant_portfolio</t>
+          <t>70% of 242 lines in 3 key file(s) run by: test_auto_recover, test_w39_quant_portfolio, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z108" s="2" t="inlineStr"/>
@@ -16274,7 +16367,7 @@
       </c>
       <c r="Y109" s="2" t="inlineStr">
         <is>
-          <t>45% of 167 lines in 2 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial, test_w39_exec_data_tests</t>
+          <t>45% of 167 lines in 2 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial, test_w39_exec_data_tests, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z109" s="2" t="inlineStr"/>
@@ -16390,7 +16483,7 @@
       </c>
       <c r="Y110" s="2" t="inlineStr">
         <is>
-          <t>87% of 423 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+55 more)</t>
+          <t>87% of 423 lines in 2 key file(s) run by: test_aggressive_lifecycle, test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_job_monitoring, test_market_health, test_mysql_backend (+65 more)</t>
         </is>
       </c>
       <c r="Z110" s="2" t="inlineStr"/>
@@ -16510,7 +16603,7 @@
       </c>
       <c r="Y111" s="2" t="inlineStr">
         <is>
-          <t>92% of 364 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_cpcv_pbo</t>
+          <t>93% of 409 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips (+1 more)</t>
         </is>
       </c>
       <c r="Z111" s="2" t="inlineStr"/>
@@ -16630,7 +16723,7 @@
       </c>
       <c r="Y112" s="2" t="inlineStr">
         <is>
-          <t>96% of 121 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_cpcv_pbo, test_w39b_mf_analytics, test_wealth_performance</t>
+          <t>96% of 121 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_mcp, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+6 more)</t>
         </is>
       </c>
       <c r="Z112" s="2" t="inlineStr"/>
@@ -16750,7 +16843,7 @@
       </c>
       <c r="Y113" s="2" t="inlineStr">
         <is>
-          <t>96% of 121 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_cpcv_pbo, test_w39b_mf_analytics, test_wealth_performance</t>
+          <t>96% of 121 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_mcp, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+6 more)</t>
         </is>
       </c>
       <c r="Z113" s="2" t="inlineStr"/>
@@ -16862,7 +16955,7 @@
       </c>
       <c r="Y114" s="2" t="inlineStr">
         <is>
-          <t>96% of 121 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_cpcv_pbo, test_w39b_mf_analytics, test_wealth_performance</t>
+          <t>96% of 121 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_mcp, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+6 more)</t>
         </is>
       </c>
       <c r="Z114" s="2" t="inlineStr"/>
@@ -16978,7 +17071,7 @@
       </c>
       <c r="Y115" s="2" t="inlineStr">
         <is>
-          <t>87% of 84 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_contract_note_fees, test_w39_performance_detail, test_w39_qa_suite, test_w39b_cpcv_pbo, test_wealth_performance (+1 more)</t>
+          <t>91% of 131 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_contract_note_fees, test_w39_performance_detail, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+7 more)</t>
         </is>
       </c>
       <c r="Z115" s="2" t="inlineStr"/>
@@ -17098,7 +17191,7 @@
       </c>
       <c r="Y116" s="2" t="inlineStr">
         <is>
-          <t>69% of 29 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_cpcv_pbo</t>
+          <t>69% of 29 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips (+1 more)</t>
         </is>
       </c>
       <c r="Z116" s="2" t="inlineStr"/>
@@ -17214,7 +17307,7 @@
       </c>
       <c r="Y117" s="2" t="inlineStr">
         <is>
-          <t>56% of 36 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_cpcv_pbo</t>
+          <t>56% of 36 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips (+1 more)</t>
         </is>
       </c>
       <c r="Z117" s="2" t="inlineStr"/>
@@ -17318,7 +17411,7 @@
       </c>
       <c r="Y118" s="2" t="inlineStr">
         <is>
-          <t>87% of 105 lines in 1 key file(s) run by: test_index_feed, test_w39_index_constituents, test_w39_perf_budget, test_w39_performance_detail, test_w39_qa_suite, test_w39_ui_smoke, test_w39b_tf75, test_wealth_api_security (+3 more)</t>
+          <t>84% of 105 lines in 1 key file(s) run by: test_index_feed, test_w39_index_constituents, test_w39_perf_budget, test_w39_performance_detail, test_w39_qa_suite, test_w39_ui_smoke, test_w39b_tf75, test_w40_total_return (+4 more)</t>
         </is>
       </c>
       <c r="Z118" s="2" t="inlineStr"/>
@@ -17438,7 +17531,7 @@
       </c>
       <c r="Y119" s="2" t="inlineStr">
         <is>
-          <t>91% of 500 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_cpcv_pbo</t>
+          <t>92% of 545 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo (+3 more)</t>
         </is>
       </c>
       <c r="Z119" s="2" t="inlineStr"/>
@@ -17558,7 +17651,7 @@
       </c>
       <c r="Y120" s="2" t="inlineStr">
         <is>
-          <t>81% of 175 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_cpcv_pbo</t>
+          <t>81% of 181 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips (+2 more)</t>
         </is>
       </c>
       <c r="Z120" s="2" t="inlineStr"/>
@@ -17678,7 +17771,7 @@
       </c>
       <c r="Y121" s="2" t="inlineStr">
         <is>
-          <t>82% of 126 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39b_cpcv_pbo</t>
+          <t>83% of 126 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z121" s="2" t="inlineStr"/>
@@ -17798,7 +17891,7 @@
       </c>
       <c r="Y122" s="2" t="inlineStr">
         <is>
-          <t>94% of 53 lines in 1 key file(s) run by: test_w39_backtest_partial, test_w39_untested_modules</t>
+          <t>94% of 53 lines in 1 key file(s) run by: test_w39_backtest_partial, test_w39_untested_modules, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z122" s="2" t="inlineStr"/>
@@ -17861,7 +17954,7 @@
       </c>
       <c r="L123" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
       <c r="M123" s="2" t="inlineStr">
@@ -17871,12 +17964,12 @@
       </c>
       <c r="N123" s="2" t="inlineStr">
         <is>
-          <t>W23: grid / random / adaptive optimiser with trial runs, test-window refusal, Deflated Sharpe + overfit warning</t>
+          <t>W23: grid / random / adaptive optimiser with trial runs, test-window refusal, Deflated Sharpe + overfit warning. W40: method="bayes" -- a Tree-structured Parzen Estimator (Bergstra et al. 2011) in numpy after a seeded random start, same trial storage and deflated-Sharpe accounting</t>
         </is>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>QA; optional true Bayesian search</t>
+          <t>Independent QA</t>
         </is>
       </c>
       <c r="P123" s="2" t="inlineStr">
@@ -17886,7 +17979,7 @@
       </c>
       <c r="Q123" s="2" t="inlineStr">
         <is>
-          <t>branch w23-research-backtest; docs/W23_RESEARCH_BACKTEST_HANDOFF.md</t>
+          <t>tests/test_w39b_bayes_optimize.py</t>
         </is>
       </c>
       <c r="R123" s="2" t="inlineStr"/>
@@ -17899,7 +17992,7 @@
       <c r="U123" s="2" t="inlineStr"/>
       <c r="V123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="W123" s="2" t="inlineStr"/>
@@ -17910,7 +18003,7 @@
       </c>
       <c r="Y123" s="2" t="inlineStr">
         <is>
-          <t>71% of 197 lines in 1 key file(s) run by: test_w39_backtest, test_w39_qa_suite, test_w39_untested_modules, test_w39b_cpcv_pbo</t>
+          <t>tests/test_w39b_bayes_optimize.py | 88% of 352 lines in 1 key file(s) run by: test_w39_backtest, test_w39_qa_suite, test_w39_untested_modules, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo</t>
         </is>
       </c>
       <c r="Z123" s="2" t="inlineStr"/>
@@ -18104,7 +18197,7 @@
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>Independent QA; the stochastic-dominance test is not implemented; CPCV runs on the W2 engine only</t>
+          <t>Independent QA. W40: first / second-order stochastic dominance of the selected trial's out-of-sample results over a random selection (in pbo() and CPCV); CPCV on the event-driven engine (engine="event_driven")</t>
         </is>
       </c>
       <c r="P125" s="2" t="inlineStr">
@@ -18114,7 +18207,7 @@
       </c>
       <c r="Q125" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_cpcv_pbo.py</t>
+          <t>tests/test_w39b_cpcv_pbo.py; tests/test_w39b_cpcv_dominance.py</t>
         </is>
       </c>
       <c r="R125" s="2" t="inlineStr"/>
@@ -18138,7 +18231,7 @@
       </c>
       <c r="Y125" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_cpcv_pbo.py | 79% of 531 lines in 2 key file(s) run by: test_w39_backtest, test_w39b_cpcv_pbo</t>
+          <t>tests/test_w39b_cpcv_pbo.py; tests/test_w39b_cpcv_dominance.py | 83% of 678 lines in 2 key file(s) run by: test_w39_backtest, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo</t>
         </is>
       </c>
       <c r="Z125" s="2" t="inlineStr"/>
@@ -18370,7 +18463,7 @@
       </c>
       <c r="Y127" s="2" t="inlineStr">
         <is>
-          <t>32% of 257 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_cpcv_pbo</t>
+          <t>43% of 259 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips (+2 more)</t>
         </is>
       </c>
       <c r="Z127" s="2" t="inlineStr"/>
@@ -18482,7 +18575,7 @@
       </c>
       <c r="Y128" s="2" t="inlineStr">
         <is>
-          <t>32% of 257 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_cpcv_pbo</t>
+          <t>43% of 259 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips (+2 more)</t>
         </is>
       </c>
       <c r="Z128" s="2" t="inlineStr"/>
@@ -18590,7 +18683,7 @@
       </c>
       <c r="Y129" s="2" t="inlineStr">
         <is>
-          <t>64% of 300 lines in 1 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_exec_data_tests, test_w39_notify_transactions, test_w39_perf_budget, test_w39_performance_detail (+5 more)</t>
+          <t>64% of 301 lines in 1 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_w39_exec_data_tests, test_w39_notify_transactions, test_w39_perf_budget, test_w39_performance_detail (+6 more)</t>
         </is>
       </c>
       <c r="Z129" s="2" t="inlineStr"/>
@@ -18926,7 +19019,7 @@
       </c>
       <c r="Y132" s="2" t="inlineStr">
         <is>
-          <t>86% of 728 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w39_untested_modules</t>
+          <t>86% of 728 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w39_technical_rs_fib, test_w39_untested_modules, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z132" s="2" t="inlineStr"/>
@@ -19046,7 +19139,7 @@
       </c>
       <c r="Y133" s="2" t="inlineStr">
         <is>
-          <t>17% of 275 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite</t>
+          <t>31% of 347 lines in 2 key file(s) run by: test_regressions, test_w37_brokers_multi_asset, test_w39_qa_suite, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z133" s="2" t="inlineStr"/>
@@ -19710,7 +19803,7 @@
       </c>
       <c r="Y139" s="2" t="inlineStr">
         <is>
-          <t>41% of 834 lines in 2 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_risk_gateway (+2 more)</t>
+          <t>40% of 834 lines in 2 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_risk_gateway (+2 more)</t>
         </is>
       </c>
       <c r="Z139" s="2" t="inlineStr"/>
@@ -20174,7 +20267,7 @@
       </c>
       <c r="Y143" s="2" t="inlineStr">
         <is>
-          <t>72% of 126 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest_partial</t>
+          <t>88% of 132 lines in 1 key file(s) run by: test_auto_recover, test_w39_backtest_partial, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z143" s="2" t="inlineStr"/>
@@ -20402,7 +20495,7 @@
       </c>
       <c r="Y145" s="2" t="inlineStr">
         <is>
-          <t>78% of 195 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial</t>
+          <t>79% of 204 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z145" s="2" t="inlineStr"/>
@@ -20522,7 +20615,7 @@
       </c>
       <c r="Y146" s="2" t="inlineStr">
         <is>
-          <t>68% of 98 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial</t>
+          <t>68% of 98 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z146" s="2" t="inlineStr"/>
@@ -20642,7 +20735,7 @@
       </c>
       <c r="Y147" s="2" t="inlineStr">
         <is>
-          <t>38% of 119 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract</t>
+          <t>58% of 119 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z147" s="2" t="inlineStr"/>
@@ -20698,9 +20791,9 @@
           <t>COMPLETED</t>
         </is>
       </c>
-      <c r="K148" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="K148" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="L148" s="2" t="inlineStr">
@@ -20762,7 +20855,7 @@
       </c>
       <c r="Y148" s="2" t="inlineStr">
         <is>
-          <t>50% of 495 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio</t>
+          <t>66% of 502 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z148" s="2" t="inlineStr"/>
@@ -20818,9 +20911,9 @@
           <t>COMPLETED</t>
         </is>
       </c>
-      <c r="K149" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="K149" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="L149" s="2" t="inlineStr">
@@ -20882,7 +20975,7 @@
       </c>
       <c r="Y149" s="2" t="inlineStr">
         <is>
-          <t>50% of 495 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio</t>
+          <t>66% of 502 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z149" s="2" t="inlineStr"/>
@@ -21002,7 +21095,7 @@
       </c>
       <c r="Y150" s="2" t="inlineStr">
         <is>
-          <t>88% of 64 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial, test_w39_exec_data_tests</t>
+          <t>88% of 64 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_backtest_partial, test_w39_exec_data_tests, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z150" s="2" t="inlineStr"/>
@@ -21478,7 +21571,7 @@
       </c>
       <c r="Y154" s="2" t="inlineStr">
         <is>
-          <t>33% of 1358 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_intraday, test_w39_notify_transactions, test_w39_qa_suite (+2 more)</t>
+          <t>33% of 1365 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_intraday, test_w39_notify_transactions, test_w39_qa_suite (+3 more)</t>
         </is>
       </c>
       <c r="Z154" s="2" t="inlineStr"/>
@@ -21710,7 +21803,7 @@
       </c>
       <c r="Y156" s="2" t="inlineStr">
         <is>
-          <t>91% of 68 lines in 2 key file(s) run by: test_w39_exec_data_tests, test_w39_perf_budget</t>
+          <t>89% of 75 lines in 2 key file(s) run by: test_w39_exec_data_tests, test_w39_perf_budget, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z156" s="2" t="inlineStr"/>
@@ -21834,7 +21927,7 @@
       </c>
       <c r="Y157" s="2" t="inlineStr">
         <is>
-          <t>76% of 104 lines in 1 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_qa_suite</t>
+          <t>76% of 106 lines in 1 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z157" s="2" t="inlineStr"/>
@@ -22074,7 +22167,7 @@
       </c>
       <c r="Y159" s="2" t="inlineStr">
         <is>
-          <t>85% of 159 lines in 1 key file(s) run by: test_auto_recover, test_w39_qa_suite</t>
+          <t>87% of 198 lines in 1 key file(s) run by: test_auto_recover, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z159" s="2" t="inlineStr"/>
@@ -22194,7 +22287,7 @@
       </c>
       <c r="Y160" s="2" t="inlineStr">
         <is>
-          <t>63% of 379 lines in 2 key file(s) run by: test_auto_recover, test_w39_qa_suite</t>
+          <t>71% of 385 lines in 2 key file(s) run by: test_auto_recover, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z160" s="2" t="inlineStr"/>
@@ -22318,7 +22411,7 @@
       </c>
       <c r="Y161" s="2" t="inlineStr">
         <is>
-          <t>70% of 178 lines in 2 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite</t>
+          <t>88% of 184 lines in 2 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z161" s="2" t="inlineStr"/>
@@ -22374,9 +22467,9 @@
           <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
-      <c r="K162" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="K162" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
@@ -22438,7 +22531,7 @@
       </c>
       <c r="Y162" s="2" t="inlineStr">
         <is>
-          <t>57% of 316 lines in 1 key file(s) run by: test_auto_recover, test_w39_qa_suite</t>
+          <t>67% of 322 lines in 1 key file(s) run by: test_auto_recover, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z162" s="2" t="inlineStr"/>
@@ -22678,7 +22771,7 @@
       </c>
       <c r="Y164" s="2" t="inlineStr">
         <is>
-          <t>67% of 475 lines in 2 key file(s) run by: test_auto_recover, test_w39_qa_suite</t>
+          <t>75% of 520 lines in 2 key file(s) run by: test_auto_recover, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z164" s="2" t="inlineStr"/>
@@ -23602,7 +23695,7 @@
       </c>
       <c r="Y172" s="2" t="inlineStr">
         <is>
-          <t>34% of 1420 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w36_ml_strategy_tooling, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite (+3 more)</t>
+          <t>34% of 1427 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w36_ml_strategy_tooling, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite (+4 more)</t>
         </is>
       </c>
       <c r="Z172" s="2" t="inlineStr"/>
@@ -23950,7 +24043,7 @@
       </c>
       <c r="Y175" s="2" t="inlineStr">
         <is>
-          <t>68% of 598 lines in 3 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite</t>
+          <t>72% of 614 lines in 3 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z175" s="2" t="inlineStr"/>
@@ -24302,7 +24395,7 @@
       </c>
       <c r="Y178" s="2" t="inlineStr">
         <is>
-          <t>36% of 484 lines in 2 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke</t>
+          <t>39% of 507 lines in 2 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z178" s="2" t="inlineStr"/>
@@ -24414,7 +24507,7 @@
       </c>
       <c r="Y179" s="2" t="inlineStr">
         <is>
-          <t>23% of 342 lines in 1 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke</t>
+          <t>29% of 365 lines in 1 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z179" s="2" t="inlineStr"/>
@@ -24534,7 +24627,7 @@
       </c>
       <c r="Y180" s="2" t="inlineStr">
         <is>
-          <t>24% of 346 lines in 2 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke</t>
+          <t>30% of 369 lines in 2 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z180" s="2" t="inlineStr"/>
@@ -24646,7 +24739,7 @@
       </c>
       <c r="Y181" s="2" t="inlineStr">
         <is>
-          <t>45% of 595 lines in 2 key file(s) run by: test_auto_recover, test_w39_risk_gateway</t>
+          <t>46% of 600 lines in 2 key file(s) run by: test_auto_recover, test_w39_risk_gateway, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z181" s="2" t="inlineStr"/>
@@ -24758,7 +24851,7 @@
       </c>
       <c r="Y182" s="2" t="inlineStr">
         <is>
-          <t>37% of 937 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>40% of 965 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_risk_gateway, test_w39_ui_smoke, test_w40_option_intents, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z182" s="2" t="inlineStr"/>
@@ -24878,7 +24971,7 @@
       </c>
       <c r="Y183" s="2" t="inlineStr">
         <is>
-          <t>51% of 604 lines in 2 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>52% of 609 lines in 2 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke, test_w40_option_intents, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z183" s="2" t="inlineStr"/>
@@ -24990,7 +25083,7 @@
       </c>
       <c r="Y184" s="2" t="inlineStr">
         <is>
-          <t>46% of 692 lines in 3 key file(s) run by: test_auto_recover, test_w38_platform_compliance, test_w39_exec_data_tests, test_w39_ops_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>47% of 697 lines in 3 key file(s) run by: test_auto_recover, test_w38_platform_compliance, test_w39_exec_data_tests, test_w39_ops_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke (+1 more)</t>
         </is>
       </c>
       <c r="Z184" s="2" t="inlineStr"/>
@@ -25102,7 +25195,7 @@
       </c>
       <c r="Y185" s="2" t="inlineStr">
         <is>
-          <t>52% of 933 lines in 3 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>53% of 938 lines in 3 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z185" s="2" t="inlineStr"/>
@@ -25222,7 +25315,7 @@
       </c>
       <c r="Y186" s="2" t="inlineStr">
         <is>
-          <t>51% of 604 lines in 2 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>52% of 609 lines in 2 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke, test_w40_option_intents, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z186" s="2" t="inlineStr"/>
@@ -25330,7 +25423,7 @@
       </c>
       <c r="Y187" s="2" t="inlineStr">
         <is>
-          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+5 more)</t>
+          <t>66% of 338 lines in 1 key file(s) run by: test_auto_recover, test_job_monitoring, test_risk_controls, test_strategy_live, test_w38_platform_compliance, test_w39_backtest, test_w39_backtest_partial, test_w39_notify_transactions (+10 more)</t>
         </is>
       </c>
       <c r="Z187" s="2" t="inlineStr"/>
@@ -25682,7 +25775,7 @@
       </c>
       <c r="Y190" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_backtest_partial.py | 73% of 1784 lines in 5 key file(s) run by: test_auto_recover, test_signal_pipeline, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_cpcv_pbo</t>
+          <t>tests/test_w39_backtest_partial.py | 79% of 1894 lines in 5 key file(s) run by: test_auto_recover, test_signal_pipeline, test_w39_backtest, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+4 more)</t>
         </is>
       </c>
       <c r="Z190" s="2" t="inlineStr"/>
@@ -25794,7 +25887,7 @@
       </c>
       <c r="Y191" s="2" t="inlineStr">
         <is>
-          <t>23% of 342 lines in 1 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke</t>
+          <t>29% of 365 lines in 1 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z191" s="2" t="inlineStr"/>
@@ -25906,7 +25999,7 @@
       </c>
       <c r="Y192" s="2" t="inlineStr">
         <is>
-          <t>23% of 342 lines in 1 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke</t>
+          <t>29% of 365 lines in 1 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z192" s="2" t="inlineStr"/>
@@ -26018,7 +26111,7 @@
       </c>
       <c r="Y193" s="2" t="inlineStr">
         <is>
-          <t>39% of 437 lines in 2 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_performance_detail, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w39b_mf_analytics, test_wealth_math (+1 more)</t>
+          <t>43% of 461 lines in 2 key file(s) run by: test_auto_recover, test_w39_mcp, test_w39_perf_budget, test_w39_performance_detail, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w39b_mf_analytics (+4 more)</t>
         </is>
       </c>
       <c r="Z193" s="2" t="inlineStr"/>
@@ -26134,7 +26227,7 @@
       </c>
       <c r="Y194" s="2" t="inlineStr">
         <is>
-          <t>100% of 4 lines in 1 key file(s) run by: test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke</t>
+          <t>100% of 4 lines in 1 key file(s) run by: test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z194" s="2" t="inlineStr"/>
@@ -26250,7 +26343,7 @@
       </c>
       <c r="Y195" s="2" t="inlineStr">
         <is>
-          <t>55% of 684 lines in 4 key file(s) run by: test_auto_recover, test_paper_broker, test_risk_controls, test_strategy_live, test_w37_brokers_multi_asset, test_w39_exec_data_tests, test_w39_performance_detail, test_w39_qa_suite (+3 more)</t>
+          <t>56% of 695 lines in 4 key file(s) run by: test_auto_recover, test_paper_broker, test_risk_controls, test_strategy_live, test_w37_brokers_multi_asset, test_w39_exec_data_tests, test_w39_performance_detail, test_w39_qa_suite (+6 more)</t>
         </is>
       </c>
       <c r="Z195" s="2" t="inlineStr"/>
@@ -26366,7 +26459,7 @@
       </c>
       <c r="Y196" s="2" t="inlineStr">
         <is>
-          <t>49% of 510 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke</t>
+          <t>52% of 542 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z196" s="2" t="inlineStr"/>
@@ -26594,7 +26687,7 @@
       </c>
       <c r="Y198" s="2" t="inlineStr">
         <is>
-          <t>73% of 135 lines in 1 key file(s) run by: test_w39_exec_data_tests, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>73% of 135 lines in 1 key file(s) run by: test_w39_exec_data_tests, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z198" s="2" t="inlineStr"/>
@@ -26714,7 +26807,7 @@
       </c>
       <c r="Y199" s="2" t="inlineStr">
         <is>
-          <t>55% of 669 lines in 2 key file(s) run by: test_auto_recover, test_w39_exec_data_tests, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>55% of 674 lines in 2 key file(s) run by: test_auto_recover, test_w39_exec_data_tests, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z199" s="2" t="inlineStr"/>
@@ -27066,7 +27159,7 @@
       </c>
       <c r="Y202" s="2" t="inlineStr">
         <is>
-          <t>100% of 78 lines in 2 key file(s) run by: test_w39_exec_data_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke</t>
+          <t>100% of 78 lines in 2 key file(s) run by: test_w39_exec_data_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z202" s="2" t="inlineStr"/>
@@ -27294,7 +27387,7 @@
       </c>
       <c r="Y204" s="2" t="inlineStr">
         <is>
-          <t>82% of 89 lines in 2 key file(s) run by: test_w39_exec_data_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke</t>
+          <t>82% of 89 lines in 2 key file(s) run by: test_w39_exec_data_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_ui_smoke, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z204" s="2" t="inlineStr"/>
@@ -27762,7 +27855,7 @@
       </c>
       <c r="Y208" s="2" t="inlineStr">
         <is>
-          <t>35% of 398 lines in 3 key file(s) run by: test_auto_recover, test_signal_pipeline, test_w39_untested_modules</t>
+          <t>38% of 398 lines in 3 key file(s) run by: test_auto_recover, test_signal_pipeline, test_w39_untested_modules, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z208" s="2" t="inlineStr"/>
@@ -27882,7 +27975,7 @@
       </c>
       <c r="Y209" s="2" t="inlineStr">
         <is>
-          <t>61% of 419 lines in 2 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio</t>
+          <t>65% of 422 lines in 2 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z209" s="2" t="inlineStr"/>
@@ -28002,7 +28095,7 @@
       </c>
       <c r="Y210" s="2" t="inlineStr">
         <is>
-          <t>12% of 208 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite</t>
+          <t>32% of 208 lines in 2 key file(s) run by: test_regressions, test_w39_qa_suite, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z210" s="2" t="inlineStr"/>
@@ -28058,14 +28151,14 @@
           <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
-      <c r="K211" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="K211" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="L211" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>90</t>
         </is>
       </c>
       <c r="M211" s="2" t="inlineStr">
@@ -28080,17 +28173,17 @@
       </c>
       <c r="O211" s="2" t="inlineStr">
         <is>
-          <t>Backtest engine does not simulate futures shorts; no auto-roll (re-entry on next signal); paper capital must exceed one lot (~Rs 5-10 lakh notional)</t>
+          <t>Independent QA. W40: the W2 backtest simulates SHORT / COVER as near-month stock futures (lots, margin, daily variation margin, NSE F&amp;O costs, a roll N sessions before expiry; refused, never priced off spot, without futures history); the paper book can auto-roll (futures.auto_roll, off by default). Not modelled: physical settlement, SPAN margin</t>
         </is>
       </c>
       <c r="P211" s="2" t="inlineStr">
         <is>
-          <t>execution/futures_paper.py; execution/risk_engine.py; execution/order_manager.py; execution/adapters.py; strategy_engine/kinds.py; strategy_engine/decisions.py</t>
+          <t>execution/futures_paper.py; backtest/futures.py; backtest/engine.py</t>
         </is>
       </c>
       <c r="Q211" s="2" t="inlineStr">
         <is>
-          <t>Scratch: SBIN 1 lot short @958.52, cover @959.48, cash -760 = realised -760; reconciliation unaffected</t>
+          <t>tests/test_w40_futures_backtest.py</t>
         </is>
       </c>
       <c r="R211" s="2" t="inlineStr">
@@ -28107,7 +28200,7 @@
       <c r="U211" s="2" t="inlineStr"/>
       <c r="V211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="W211" s="2" t="inlineStr">
@@ -28122,7 +28215,7 @@
       </c>
       <c r="Y211" s="2" t="inlineStr">
         <is>
-          <t>50% of 1704 lines in 6 key file(s) run by: test_auto_recover, test_risk_controls, test_signal_pipeline, test_w39_backtest_partial, test_w39_exec_data_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio (+2 more)</t>
+          <t>tests/test_w40_futures_backtest.py | 90% of 1065 lines in 3 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_backtest, test_w39_backtest_partial, test_w39_exec_data_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway (+7 more)</t>
         </is>
       </c>
       <c r="Z211" s="2" t="inlineStr"/>
@@ -28178,9 +28271,9 @@
           <t>IMPLEMENTED BUT NOT VERIFIED</t>
         </is>
       </c>
-      <c r="K212" s="15" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="K212" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="L212" s="2" t="inlineStr">
@@ -28200,7 +28293,7 @@
       </c>
       <c r="O212" s="2" t="inlineStr">
         <is>
-          <t>Same limits as QR-05; lot granularity makes small books non-neutral -- check exposure after sizing</t>
+          <t>Independent QA. W40: long/short portfolios backtest with their futures legs (see QR-05); lot granularity still makes small books non-neutral -- check exposure after sizing</t>
         </is>
       </c>
       <c r="P212" s="2" t="inlineStr">
@@ -28210,7 +28303,7 @@
       </c>
       <c r="Q212" s="2" t="inlineStr">
         <is>
-          <t>Compile + definition validation</t>
+          <t>tests/test_w40_futures_backtest.py</t>
         </is>
       </c>
       <c r="R212" s="2" t="inlineStr">
@@ -28227,7 +28320,7 @@
       <c r="U212" s="2" t="inlineStr"/>
       <c r="V212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="W212" s="2" t="inlineStr">
@@ -28242,7 +28335,7 @@
       </c>
       <c r="Y212" s="2" t="inlineStr">
         <is>
-          <t>50% of 495 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio</t>
+          <t>tests/test_w40_futures_backtest.py | 66% of 502 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_backtest_partial, test_w39_qa_suite, test_w39_quant_portfolio, test_w39b_event_driven_skips, test_w40_futures_backtest, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z212" s="2" t="inlineStr"/>
@@ -28362,7 +28455,7 @@
       </c>
       <c r="Y213" s="2" t="inlineStr">
         <is>
-          <t>5% of 258 lines in 4 key file(s) run by: test_auto_recover, test_signal_pipeline</t>
+          <t>11% of 258 lines in 4 key file(s) run by: test_auto_recover, test_signal_pipeline, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z213" s="2" t="inlineStr"/>
@@ -28482,7 +28575,7 @@
       </c>
       <c r="Y214" s="2" t="inlineStr">
         <is>
-          <t>61% of 266 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio</t>
+          <t>68% of 269 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z214" s="2" t="inlineStr"/>
@@ -28598,7 +28691,7 @@
       </c>
       <c r="Y215" s="2" t="inlineStr">
         <is>
-          <t>11% of 466 lines in 3 key file(s) run by: test_auto_recover</t>
+          <t>29% of 466 lines in 3 key file(s) run by: test_auto_recover, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z215" s="2" t="inlineStr"/>
@@ -28714,7 +28807,7 @@
       </c>
       <c r="Y216" s="2" t="inlineStr">
         <is>
-          <t>71% of 101 lines in 1 key file(s) run by: test_w39_backtest_partial, test_w39_performance_detail, test_w39_untested_modules</t>
+          <t>71% of 101 lines in 1 key file(s) run by: test_w39_backtest_partial, test_w39_performance_detail, test_w39_untested_modules, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z216" s="2" t="inlineStr"/>
@@ -28826,7 +28919,7 @@
       </c>
       <c r="Y217" s="2" t="inlineStr">
         <is>
-          <t>50% of 1316 lines in 4 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live (+5 more)</t>
+          <t>50% of 1327 lines in 4 key file(s) run by: test_auto_recover, test_corporate_actions, test_fii_dii_and_delivery_factor, test_index_feed, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live (+6 more)</t>
         </is>
       </c>
       <c r="Z217" s="2" t="inlineStr"/>
@@ -28942,7 +29035,7 @@
       </c>
       <c r="Y218" s="2" t="inlineStr">
         <is>
-          <t>34% of 407 lines in 3 key file(s) run by: test_auto_recover</t>
+          <t>36% of 418 lines in 3 key file(s) run by: test_auto_recover, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z218" s="2" t="inlineStr"/>
@@ -29020,7 +29113,7 @@
       </c>
       <c r="O219" s="2" t="inlineStr">
         <is>
-          <t>Independent QA; the engine does not yet report the adapter's skipped decisions the way W2 does</t>
+          <t>Independent QA. W40: reports the adapter's skipped decisions like W2; fix: the end-of-window close-out is now in the last day's return (chained returns overstated final equity by the close-out costs). It still does not trade SHORT (W2 does, as futures)</t>
         </is>
       </c>
       <c r="P219" s="2" t="inlineStr">
@@ -29030,7 +29123,7 @@
       </c>
       <c r="Q219" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_backtest_partial.py (test_event_driven_*)</t>
+          <t>tests/test_w39_backtest_partial.py (test_event_driven_*); tests/test_w39b_event_driven_skips.py</t>
         </is>
       </c>
       <c r="R219" s="2" t="inlineStr"/>
@@ -29058,7 +29151,7 @@
       </c>
       <c r="Y219" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_backtest_partial.py (test_event_driven_*) | 79% of 532 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest_partial</t>
+          <t>tests/test_w39_backtest_partial.py (test_event_driven_*); tests/test_w39b_event_driven_skips.py | 81% of 568 lines in 2 key file(s) run by: test_auto_recover, test_w39_backtest_partial, test_w39b_cpcv_dominance, test_w39b_event_driven_skips, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z219" s="2" t="inlineStr"/>
@@ -30434,7 +30527,7 @@
       </c>
       <c r="Y231" s="2" t="inlineStr">
         <is>
-          <t>49% of 377 lines in 3 key file(s) run by: test_auto_recover, test_w37_brokers_multi_asset, test_w39_api_contract, test_w39_depth20, test_w39_risk_gateway</t>
+          <t>51% of 403 lines in 3 key file(s) run by: test_auto_recover, test_w37_brokers_multi_asset, test_w39_api_contract, test_w39_depth20, test_w39_risk_gateway, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z231" s="2" t="inlineStr"/>
@@ -30550,7 +30643,7 @@
       </c>
       <c r="Y232" s="2" t="inlineStr">
         <is>
-          <t>67% of 486 lines in 4 key file(s) run by: test_mysql_backend, test_postgres_backend, test_w38_platform_compliance, test_w39_perf_budget, test_w39b_razorpay</t>
+          <t>69% of 531 lines in 4 key file(s) run by: test_mysql_backend, test_postgres_backend, test_w36_ml_strategy_tooling, test_w38_platform_compliance, test_w39_perf_budget, test_w39b_razorpay</t>
         </is>
       </c>
       <c r="Z232" s="2" t="inlineStr"/>
@@ -31154,7 +31247,7 @@
       </c>
       <c r="Y237" s="2" t="inlineStr">
         <is>
-          <t>46% of 757 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_risk_gateway, test_w39b_razorpay</t>
+          <t>47% of 762 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_risk_gateway, test_w39b_razorpay, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z237" s="2" t="inlineStr"/>
@@ -31618,7 +31711,7 @@
       </c>
       <c r="Y241" s="2" t="inlineStr">
         <is>
-          <t>48% of 231 lines in 2 key file(s) run by: test_auto_recover, test_w38_platform_compliance, test_w39_depth20, test_w39_event_calendar, test_w39_global_sync, test_w39_intraday, test_w39_market_pulse, test_w39_perf_budget (+8 more)</t>
+          <t>48% of 231 lines in 2 key file(s) run by: test_auto_recover, test_w38_platform_compliance, test_w39_depth20, test_w39_event_calendar, test_w39_global_sync, test_w39_intraday, test_w39_market_pulse, test_w39_perf_budget (+10 more)</t>
         </is>
       </c>
       <c r="Z241" s="2" t="inlineStr"/>
@@ -32342,7 +32435,7 @@
       </c>
       <c r="Y247" s="2" t="inlineStr">
         <is>
-          <t>33% of 1430 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+1 more)</t>
+          <t>33% of 1437 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_qa_suite, test_w39_ui_smoke (+2 more)</t>
         </is>
       </c>
       <c r="Z247" s="2" t="inlineStr"/>
@@ -32582,7 +32675,7 @@
       </c>
       <c r="Y249" s="2" t="inlineStr">
         <is>
-          <t>test_a_deprecated_v1_resource_warns_then_answers_410_after_sunset | 59% of 657 lines in 3 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+27 more)</t>
+          <t>test_a_deprecated_v1_resource_warns_then_answers_410_after_sunset | 59% of 657 lines in 3 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+34 more)</t>
         </is>
       </c>
       <c r="Z249" s="2" t="inlineStr"/>
@@ -32997,7 +33090,7 @@
       </c>
       <c r="L253" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>85</t>
         </is>
       </c>
       <c r="M253" s="2" t="inlineStr">
@@ -33012,17 +33105,17 @@
       </c>
       <c r="O253" s="2" t="inlineStr">
         <is>
-          <t>Owner: options.enabled; QA; strategies do not emit option intents yet</t>
+          <t>Owner: options.enabled; QA. W40: option-overlay strategies (strategy_engine/option_overlay.py) emit multi-leg OPTION intents -- covered call, protective put, spreads, iron condor and more, strikes by delta or % OTM, monthly expiry -- sized by the risk engine (max loss, margin approximation, naked short calls refused unless allowed), filled all-or-nothing in the paper options book, marked daily, exited by rule, settled at expiry; PAPER only, LIVE refused; a replay on stored daily option prices</t>
         </is>
       </c>
       <c r="P253" s="2" t="inlineStr">
         <is>
-          <t>execution/options_paper.py; execution/assets.py</t>
+          <t>execution/options_paper.py; execution/option_intents.py; strategy_engine/option_overlay.py</t>
         </is>
       </c>
       <c r="Q253" s="2" t="inlineStr">
         <is>
-          <t>BRD-001</t>
+          <t>tests/test_w40_option_intents.py; docs/W40_OPTION_INTENTS_HANDOFF.md</t>
         </is>
       </c>
       <c r="R253" s="2" t="inlineStr"/>
@@ -33035,7 +33128,7 @@
       <c r="U253" s="2" t="inlineStr"/>
       <c r="V253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="W253" s="2" t="inlineStr">
@@ -33050,7 +33143,7 @@
       </c>
       <c r="Y253" s="2" t="inlineStr">
         <is>
-          <t>75% of 167 lines in 2 key file(s) run by: test_w37_brokers_multi_asset</t>
+          <t>tests/test_w40_option_intents.py; docs/W40_OPTION_INTENTS_HANDOFF.md | 84% of 1203 lines in 3 key file(s) run by: test_signal_pipeline, test_w37_brokers_multi_asset, test_w39_exec_data_tests, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z253" s="2" t="inlineStr"/>
@@ -33874,7 +33967,7 @@
       </c>
       <c r="Y260" s="2" t="inlineStr">
         <is>
-          <t>71% of 254 lines in 1 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+27 more)</t>
+          <t>71% of 254 lines in 1 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+34 more)</t>
         </is>
       </c>
       <c r="Z260" s="2" t="inlineStr"/>
@@ -33990,7 +34083,7 @@
       </c>
       <c r="Y261" s="2" t="inlineStr">
         <is>
-          <t>53% of 232 lines in 2 key file(s) run by: test_auto_recover, test_regressions, test_risk_controls, test_w38_platform_compliance, test_w39_api_contract, test_w39_backtest, test_w39_delivery, test_w39_depth20 (+31 more)</t>
+          <t>53% of 232 lines in 2 key file(s) run by: test_auto_recover, test_regressions, test_risk_controls, test_w38_platform_compliance, test_w39_api_contract, test_w39_backtest, test_w39_delivery, test_w39_depth20 (+37 more)</t>
         </is>
       </c>
       <c r="Z261" s="2" t="inlineStr"/>
@@ -34106,7 +34199,7 @@
       </c>
       <c r="Y262" s="2" t="inlineStr">
         <is>
-          <t>36% of 1350 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_ops_tests, test_w39_perf_budget (+3 more)</t>
+          <t>35% of 1357 lines in 2 key file(s) run by: test_auto_recover, test_fii_dii_and_delivery_factor, test_job_monitoring, test_signal_pipeline, test_w39_history, test_w39_notify_transactions, test_w39_ops_tests, test_w39_perf_budget (+4 more)</t>
         </is>
       </c>
       <c r="Z262" s="2" t="inlineStr"/>
@@ -34222,7 +34315,7 @@
       </c>
       <c r="Y263" s="2" t="inlineStr">
         <is>
-          <t>32% of 1132 lines in 4 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_risk_gateway (+2 more)</t>
+          <t>31% of 1132 lines in 4 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_risk_gateway (+2 more)</t>
         </is>
       </c>
       <c r="Z263" s="2" t="inlineStr"/>
@@ -34454,7 +34547,7 @@
       </c>
       <c r="Y265" s="2" t="inlineStr">
         <is>
-          <t>50% of 880 lines in 3 key file(s) run by: test_auto_recover, test_w38_platform_compliance, test_w39_exec_data_tests, test_w39_ops_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke</t>
+          <t>51% of 896 lines in 3 key file(s) run by: test_auto_recover, test_w38_platform_compliance, test_w39_exec_data_tests, test_w39_ops_tests, test_w39_perf_budget, test_w39_qa_suite, test_w39_risk_gateway, test_w39_ui_smoke (+1 more)</t>
         </is>
       </c>
       <c r="Z265" s="2" t="inlineStr"/>
@@ -35378,7 +35471,7 @@
       </c>
       <c r="Y273" s="2" t="inlineStr">
         <is>
-          <t>89% of 1179 lines in 6 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_performance_detail, test_w39b_mf_analytics, test_wealth_api_security, test_wealth_math, test_wealth_performance (+1 more)</t>
+          <t>90% of 1207 lines in 6 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_mcp, test_w39_notify_transactions, test_w39_performance_detail, test_w39b_mf_analytics, test_w40_total_return, test_wealth_api_security (+3 more)</t>
         </is>
       </c>
       <c r="Z273" s="2" t="inlineStr"/>
@@ -35726,7 +35819,7 @@
       </c>
       <c r="Y276" s="2" t="inlineStr">
         <is>
-          <t>75% of 204 lines in 2 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+27 more)</t>
+          <t>75% of 204 lines in 2 key file(s) run by: test_auto_recover, test_risk_controls, test_w39_api_contract, test_w39_backtest, test_w39_depth20, test_w39_event_calendar, test_w39_exec_data_tests, test_w39_global_sync (+34 more)</t>
         </is>
       </c>
       <c r="Z276" s="2" t="inlineStr"/>
@@ -36074,7 +36167,7 @@
       </c>
       <c r="Y279" s="2" t="inlineStr">
         <is>
-          <t>test_paper_partial_fills_reach_the_ledger; test_entry_order_is_portable_and_numbered; test_migration_0006_numbers_old_rows_and_the_ledger_stays_append_only; test_cash_rows_and_fee_breakdown_are_validated; test_voided_transactions_are_ignored_but_kept | 77% of 317 lines in 3 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_ops_tests, test_w39_perf_budget, test_w39_performance_detail, test_wealth_api_security, test_wealth_performance (+1 more)</t>
+          <t>test_paper_partial_fills_reach_the_ledger; test_entry_order_is_portable_and_numbered; test_migration_0006_numbers_old_rows_and_the_ledger_stays_append_only; test_cash_rows_and_fee_breakdown_are_validated; test_voided_transactions_are_ignored_but_kept | 77% of 317 lines in 3 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_ops_tests, test_w39_perf_budget, test_w39_performance_detail, test_w40_total_return, test_wealth_api_security (+2 more)</t>
         </is>
       </c>
       <c r="Z279" s="2" t="inlineStr"/>
@@ -36190,7 +36283,7 @@
       </c>
       <c r="Y280" s="2" t="inlineStr">
         <is>
-          <t>test_model_return_is_reproducible_and_matches_a_hand_calculation; test_model_and_executable_are_reported_separately | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_model_return_is_reproducible_and_matches_a_hand_calculation; test_model_and_executable_are_reported_separately | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z280" s="2" t="inlineStr"/>
@@ -36306,7 +36399,7 @@
       </c>
       <c r="Y281" s="2" t="inlineStr">
         <is>
-          <t>test_executable_applies_slippage_costs_and_the_liquidity_cap; test_impact_slippage_uses_the_square_root_estimate_known_at_the_signal | 83% of 331 lines in 2 key file(s) run by: test_w39_backtest_partial, test_w39_contract_note_fees, test_w39_performance_detail, test_w39_untested_modules, test_wealth_performance</t>
+          <t>test_executable_applies_slippage_costs_and_the_liquidity_cap; test_impact_slippage_uses_the_square_root_estimate_known_at_the_signal | 83% of 331 lines in 2 key file(s) run by: test_w39_backtest_partial, test_w39_contract_note_fees, test_w39_performance_detail, test_w39_untested_modules, test_w40_futures_backtest, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z281" s="2" t="inlineStr"/>
@@ -36422,7 +36515,7 @@
       </c>
       <c r="Y282" s="2" t="inlineStr">
         <is>
-          <t>test_period_scope_is_separate_from_lifetime; test_xirr_and_pme_match_hand_computed_flows; test_average_cost_realized_pnl_and_fees | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_period_scope_is_separate_from_lifetime; test_xirr_and_pme_match_hand_computed_flows; test_average_cost_realized_pnl_and_fees | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z282" s="2" t="inlineStr"/>
@@ -36491,22 +36584,22 @@
       <c r="M283" s="2" t="inlineStr"/>
       <c r="N283" s="2" t="inlineStr">
         <is>
-          <t>any prices_daily symbol (NIFTY50, NIFTYBANK, midcap, smallcap, sector indices); price return over the same sessions + PME of the investor's flows; W39: days invested shown and exported</t>
+          <t>any prices_daily symbol (NIFTY50, NIFTYBANK, midcap, smallcap, sector indices); price return over the same sessions + PME of the investor's flows; W39: days invested shown and exported. W40: benchmark "nifty50tr" -- the Nifty 50 with dividends reinvested (data/total_return.py: NSE's TRI method, the price index exact, its dividend points estimated from the top 50 stored stocks by cap, picked monthly and weighted daily; nightly 21:10; GET /api/data/total-return), part of the report's audited inputs</t>
         </is>
       </c>
       <c r="O283" s="2" t="inlineStr">
         <is>
-          <t>Total-return index (dividends) not available from the data source</t>
+          <t>Independent QA; the dividend part is an estimate (no free-float or constituent data) -- compare once with NSE's published TRI</t>
         </is>
       </c>
       <c r="P283" s="2" t="inlineStr">
         <is>
-          <t>wealth/perf/data.py; wealth/perf/report.py</t>
+          <t>wealth/perf/data.py; wealth/perf/report.py; data/total_return.py</t>
         </is>
       </c>
       <c r="Q283" s="2" t="inlineStr">
         <is>
-          <t>test_benchmark_return_is_the_price_return_over_the_sessions</t>
+          <t>test_benchmark_return_is_the_price_return_over_the_sessions; tests/test_w40_total_return.py</t>
         </is>
       </c>
       <c r="R283" s="2" t="inlineStr">
@@ -36538,7 +36631,7 @@
       </c>
       <c r="Y283" s="2" t="inlineStr">
         <is>
-          <t>test_benchmark_return_is_the_price_return_over_the_sessions | 93% of 299 lines in 2 key file(s) run by: test_w39_performance_detail, test_w39b_mf_analytics, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_benchmark_return_is_the_price_return_over_the_sessions; tests/test_w40_total_return.py | 91% of 502 lines in 3 key file(s) run by: test_w39_mcp, test_w39_performance_detail, test_w39b_mf_analytics, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z283" s="2" t="inlineStr"/>
@@ -36654,7 +36747,7 @@
       </c>
       <c r="Y284" s="2" t="inlineStr">
         <is>
-          <t>test_costs_reconcile_with_dividend_tax_fee_rows_and_a_capped_sell; test_statutory_estimate_itemises_paper_brokerage_only_trades; tests/test_w39_contract_note_fees.py | 89% of 587 lines in 2 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_costs_reconcile_with_dividend_tax_fee_rows_and_a_capped_sell; test_statutory_estimate_itemises_paper_brokerage_only_trades; tests/test_w39_contract_note_fees.py | 89% of 587 lines in 2 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z284" s="2" t="inlineStr"/>
@@ -36770,7 +36863,7 @@
       </c>
       <c r="Y285" s="2" t="inlineStr">
         <is>
-          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win; test_position_attribution_identity | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win; test_position_attribution_identity | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z285" s="2" t="inlineStr"/>
@@ -36886,7 +36979,7 @@
       </c>
       <c r="Y286" s="2" t="inlineStr">
         <is>
-          <t>test_risk_metrics_match_independent_formulas; test_cagr_annualises_a_full_year; test_xirr_one_year_ten_percent; test_trade_stats | 96% of 216 lines in 2 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_cpcv_pbo, test_w39b_mf_analytics, test_wealth_math (+1 more)</t>
+          <t>test_risk_metrics_match_independent_formulas; test_cagr_annualises_a_full_year; test_xirr_one_year_ten_percent; test_trade_stats | 96% of 217 lines in 2 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_mcp, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+7 more)</t>
         </is>
       </c>
       <c r="Z286" s="2" t="inlineStr"/>
@@ -37002,7 +37095,7 @@
       </c>
       <c r="Y287" s="2" t="inlineStr">
         <is>
-          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win | 92% of 461 lines in 2 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win | 92% of 461 lines in 2 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z287" s="2" t="inlineStr"/>
@@ -37118,7 +37211,7 @@
       </c>
       <c r="Y288" s="2" t="inlineStr">
         <is>
-          <t>test_risk_contribution_reconciles_and_groups_sum_to_the_total; test_contributions_reconcile_to_the_total | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_risk_contribution_reconciles_and_groups_sum_to_the_total; test_contributions_reconcile_to_the_total | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z288" s="2" t="inlineStr"/>
@@ -37350,7 +37443,7 @@
       </c>
       <c r="Y290" s="2" t="inlineStr">
         <is>
-          <t>test_verify_reproduces_and_detects_changed_inputs | 95% of 231 lines in 1 key file(s) run by: test_w39_performance_detail, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_verify_reproduces_and_detects_changed_inputs | 96% of 231 lines in 1 key file(s) run by: test_w39_performance_detail, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z290" s="2" t="inlineStr"/>
@@ -37466,7 +37559,7 @@
       </c>
       <c r="Y291" s="2" t="inlineStr">
         <is>
-          <t>test_export_carries_every_section_with_the_reports_numbers; test_strategy_filter_limits_the_actual_portfolio; test_printable_html_has_the_csv_sections_and_numbers_and_escapes_text | 87% of 594 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_performance_detail, test_w39_ui_smoke, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_export_carries_every_section_with_the_reports_numbers; test_strategy_filter_limits_the_actual_portfolio; test_printable_html_has_the_csv_sections_and_numbers_and_escapes_text | 87% of 594 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_performance_detail, test_w39_ui_smoke, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z291" s="2" t="inlineStr"/>
@@ -37582,7 +37675,7 @@
       </c>
       <c r="Y292" s="2" t="inlineStr">
         <is>
-          <t>test_a_trade_on_a_market_holiday_counts_on_the_next_session; test_missing_bars_are_reported_not_hidden; test_a_bonus_issue_keeps_value_and_cost; test_an_opening_position_is_measured_from_that_days_close; test_split_between_buy_and_today_moves_neither_value_nor_return | 89% of 1179 lines in 6 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_performance_detail, test_w39b_mf_analytics, test_wealth_api_security, test_wealth_math, test_wealth_performance (+1 more)</t>
+          <t>test_a_trade_on_a_market_holiday_counts_on_the_next_session; test_missing_bars_are_reported_not_hidden; test_a_bonus_issue_keeps_value_and_cost; test_an_opening_position_is_measured_from_that_days_close; test_split_between_buy_and_today_moves_neither_value_nor_return | 90% of 1207 lines in 6 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_mcp, test_w39_notify_transactions, test_w39_performance_detail, test_w39b_mf_analytics, test_w40_total_return, test_wealth_api_security (+3 more)</t>
         </is>
       </c>
       <c r="Z292" s="2" t="inlineStr"/>
@@ -37814,7 +37907,7 @@
       </c>
       <c r="Y294" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_history.py; tests/test_w39b_merge.py | 51% of 1001 lines in 3 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_ops_tests (+3 more)</t>
+          <t>tests/test_w39_history.py; tests/test_w39b_merge.py | 50% of 1001 lines in 3 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_ops_tests (+3 more)</t>
         </is>
       </c>
       <c r="Z294" s="2" t="inlineStr"/>
@@ -37883,7 +37976,7 @@
       <c r="M295" s="2" t="inlineStr"/>
       <c r="N295" s="2" t="inlineStr">
         <is>
-          <t>W26 stock panel + W39: 3Y / 5Y / All, daily / weekly / monthly bars, SMA 20/50/200, EMA 21, Bollinger, log scale, multi-year returns; checked in headless Chromium</t>
+          <t>W26 stock panel + W39: 3Y / 5Y / All, daily / weekly / monthly bars, SMA 20/50/200, EMA 21, Bollinger, log scale, multi-year returns; checked in headless Chromium. W39b: signal / pattern marks. W40: RSI 14 and MACD 12-26-9 panels (the server's definitions), an intraday chart (1D / 5D on 15-minute bars, session VWAP, previous close, intraday scan marks; GET /api/stock/{symbol}/intraday) and the on-demand 75-minute rating</t>
         </is>
       </c>
       <c r="O295" s="2" t="inlineStr">
@@ -37898,7 +37991,7 @@
       </c>
       <c r="Q295" s="2" t="inlineStr">
         <is>
-          <t>test_stock_history_reports_multi_year_returns</t>
+          <t>test_stock_history_reports_multi_year_returns; tests/test_w40_stock_chart.py</t>
         </is>
       </c>
       <c r="R295" s="2" t="inlineStr">
@@ -37930,7 +38023,7 @@
       </c>
       <c r="Y295" s="2" t="inlineStr">
         <is>
-          <t>test_stock_history_reports_multi_year_returns | 84% of 113 lines in 1 key file(s) run by: test_auto_recover, test_w39_owner_notes, test_w39_perf_budget, test_w39b_patterns_more</t>
+          <t>test_stock_history_reports_multi_year_returns; tests/test_w40_stock_chart.py | 88% of 248 lines in 1 key file(s) run by: test_auto_recover, test_w39_mcp, test_w39_owner_notes, test_w39_perf_budget, test_w39b_patterns_more, test_w39b_tf75_signals, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z295" s="2" t="inlineStr"/>
@@ -38046,7 +38139,7 @@
       </c>
       <c r="Y296" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_risk_gateway.py | 51% of 1617 lines in 3 key file(s) run by: test_auto_recover, test_corporate_actions, test_job_monitoring, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w38_platform_compliance (+10 more)</t>
+          <t>tests/test_w39_risk_gateway.py | 51% of 1622 lines in 3 key file(s) run by: test_auto_recover, test_corporate_actions, test_job_monitoring, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w38_platform_compliance (+15 more)</t>
         </is>
       </c>
       <c r="Z296" s="2" t="inlineStr"/>
@@ -38162,7 +38255,7 @@
       </c>
       <c r="Y297" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_quant_portfolio.py | 61% of 266 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio</t>
+          <t>tests/test_w39_quant_portfolio.py | 68% of 269 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z297" s="2" t="inlineStr"/>
@@ -38510,7 +38603,7 @@
       </c>
       <c r="Y300" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_ml_regime_lineage_surface.py | 86% of 140 lines in 1 key file(s) run by: test_w36_ml_strategy_tooling, test_w39_ml_regime_lineage_surface, test_w39_options</t>
+          <t>tests/test_w39_ml_regime_lineage_surface.py | 86% of 140 lines in 1 key file(s) run by: test_w36_ml_strategy_tooling, test_w39_ml_regime_lineage_surface, test_w39_options, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z300" s="2" t="inlineStr"/>
@@ -38626,7 +38719,7 @@
       </c>
       <c r="Y301" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_ml_regime_lineage_surface.py | 87% of 341 lines in 2 key file(s) run by: test_w39_ml_regime_lineage_surface</t>
+          <t>tests/test_w39_ml_regime_lineage_surface.py | 87% of 341 lines in 2 key file(s) run by: test_w39_ml_regime_lineage_surface, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z301" s="2" t="inlineStr"/>
@@ -38742,7 +38835,7 @@
       </c>
       <c r="Y302" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_ml_regime_lineage_surface.py | 73% of 148 lines in 1 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite</t>
+          <t>tests/test_w39_ml_regime_lineage_surface.py | 88% of 154 lines in 1 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z302" s="2" t="inlineStr"/>
@@ -38858,7 +38951,7 @@
       </c>
       <c r="Y303" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_backtest.py | 82% of 126 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39b_cpcv_pbo</t>
+          <t>tests/test_w39_backtest.py | 83% of 126 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z303" s="2" t="inlineStr"/>
@@ -39898,7 +39991,7 @@
       </c>
       <c r="Y312" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_options.py | 88% of 209 lines in 1 key file(s) run by: test_w39_options</t>
+          <t>tests/test_w39_options.py | 88% of 209 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_options, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z312" s="2" t="inlineStr"/>
@@ -40014,7 +40107,7 @@
       </c>
       <c r="Y313" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_technicals.py | 88% of 820 lines in 2 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+9 more)</t>
+          <t>tests/test_w39_technicals.py | 89% of 885 lines in 2 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+12 more)</t>
         </is>
       </c>
       <c r="Z313" s="2" t="inlineStr"/>
@@ -40246,7 +40339,7 @@
       </c>
       <c r="Y315" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_regime_gate.py | 83% of 248 lines in 1 key file(s) run by: test_w39_delivery, test_w39_event_calendar, test_w39_market_pulse, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_regime_gate.py | 83% of 248 lines in 1 key file(s) run by: test_w39_delivery, test_w39_event_calendar, test_w39_market_pulse, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_technicals (+6 more)</t>
         </is>
       </c>
       <c r="Z315" s="2" t="inlineStr"/>
@@ -40362,7 +40455,7 @@
       </c>
       <c r="Y316" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_track_record.py | 84% of 522 lines in 1 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+6 more)</t>
+          <t>tests/test_w39_track_record.py | 85% of 587 lines in 1 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+9 more)</t>
         </is>
       </c>
       <c r="Z316" s="2" t="inlineStr"/>
@@ -40478,7 +40571,7 @@
       </c>
       <c r="Y317" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_weekly.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_weekly.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z317" s="2" t="inlineStr"/>
@@ -40594,7 +40687,7 @@
       </c>
       <c r="Y318" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_patterns.py; tests/test_w39b_patterns_more.py | 93% of 491 lines in 2 key file(s) run by: test_auto_recover, test_w39_delivery, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_patterns.py; tests/test_w39b_patterns_more.py | 93% of 626 lines in 2 key file(s) run by: test_auto_recover, test_w39_delivery, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z318" s="2" t="inlineStr"/>
@@ -40710,7 +40803,7 @@
       </c>
       <c r="Y319" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_rs_line.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_rs_line.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z319" s="2" t="inlineStr"/>
@@ -40826,7 +40919,7 @@
       </c>
       <c r="Y320" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_delivery.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_delivery.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z320" s="2" t="inlineStr"/>
@@ -41174,7 +41267,7 @@
       </c>
       <c r="Y323" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_intraday.py | 88% of 225 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals, test_w39_weekly, test_w39b_tf75</t>
+          <t>tests/test_w39_intraday.py | 88% of 225 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals, test_w39_weekly, test_w39b_tf75 (+2 more)</t>
         </is>
       </c>
       <c r="Z323" s="2" t="inlineStr"/>
@@ -41591,7 +41684,7 @@
       <c r="M327" s="2" t="inlineStr"/>
       <c r="N327" s="2" t="inlineStr">
         <is>
-          <t>tools/atip_mcp.py</t>
+          <t>tools/atip_mcp.py; W40: 20 tools -- adds dvm, earnings_surprise, mf_search / mf_analytics / mf_sip / mf_compare, backtest_validation (stored CPCV / PBO) and chart_marks, each checked under query_only</t>
         </is>
       </c>
       <c r="O327" s="2" t="inlineStr">
@@ -41638,7 +41731,7 @@
       </c>
       <c r="Y327" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_mcp.py | 83% of 184 lines in 1 key file(s) run by: test_w39_mcp</t>
+          <t>tests/test_w39_mcp.py | 91% of 331 lines in 1 key file(s) run by: test_w39_mcp</t>
         </is>
       </c>
       <c r="Z327" s="2" t="inlineStr"/>
@@ -41828,7 +41921,7 @@
       </c>
       <c r="O329" s="2" t="inlineStr">
         <is>
-          <t>Independent QA; no live intraday refresh (once a day, as of the close); /signals has no 75-minute column</t>
+          <t>Independent QA. W40: a 75m column on /signals and GET /api/stock/{symbol}/rating-75 (on demand from the stored 15-minute bars, completed bars only); the /signals column is still the 20:30 snapshot</t>
         </is>
       </c>
       <c r="P329" s="2" t="inlineStr">
@@ -41838,7 +41931,7 @@
       </c>
       <c r="Q329" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_tf75.py</t>
+          <t>tests/test_w39b_tf75.py; tests/test_w39b_tf75_signals.py</t>
         </is>
       </c>
       <c r="R329" s="2" t="inlineStr">
@@ -41870,7 +41963,7 @@
       </c>
       <c r="Y329" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_tf75.py | 88% of 1266 lines in 3 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+10 more)</t>
+          <t>tests/test_w39b_tf75.py; tests/test_w39b_tf75_signals.py | 89% of 1331 lines in 3 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+13 more)</t>
         </is>
       </c>
       <c r="Z329" s="2" t="inlineStr"/>
@@ -41986,7 +42079,7 @@
       </c>
       <c r="Y330" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_dvm.py | 86% of 1041 lines in 3 key file(s) run by: test_auto_recover, test_w39_depth20, test_w39_event_calendar, test_w39_global_sync, test_w39_intraday, test_w39_market_pulse, test_w39_mcp, test_w39_options (+12 more)</t>
+          <t>tests/test_w39b_dvm.py | 86% of 1044 lines in 3 key file(s) run by: test_auto_recover, test_w39_depth20, test_w39_event_calendar, test_w39_global_sync, test_w39_intraday, test_w39_market_pulse, test_w39_mcp, test_w39_options (+14 more)</t>
         </is>
       </c>
       <c r="Z330" s="2" t="inlineStr"/>
@@ -42102,7 +42195,7 @@
       </c>
       <c r="Y331" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_earnings_surprise.py | 85% of 905 lines in 2 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+6 more)</t>
+          <t>tests/test_w39b_earnings_surprise.py | 86% of 970 lines in 2 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+9 more)</t>
         </is>
       </c>
       <c r="Z331" s="2" t="inlineStr">
@@ -42175,12 +42268,12 @@
       <c r="M332" s="2" t="inlineStr"/>
       <c r="N332" s="2" t="inlineStr">
         <is>
-          <t>data/mf_analytics.py: point-to-point and CAGR returns, 1Y / 3Y rolling returns with hurdle stats, volatility / Sharpe / Sortino, drawdown with dates, beta / alpha / tracking error vs a price index, SIP and lump-sum XIRR, category rank among stored schemes, side-by-side compare; 3 read-only GET routes; scheme detail card on /data-platform</t>
+          <t>data/mf_analytics.py: point-to-point and CAGR returns, 1Y / 3Y rolling returns with hurdle stats, volatility / Sharpe / Sortino, drawdown with dates, beta / alpha / tracking error vs a price index, SIP and lump-sum XIRR, category rank among stored schemes, side-by-side compare; 3 read-only GET routes; scheme detail card on /data-platform. W40: step-up SIP, stamp duty (0.005 %) and units rounded down to 3 decimals by default, optional flat exit load per instalment; volatility annualised by the NAVs actually observed a year (not a fixed 252)</t>
         </is>
       </c>
       <c r="O332" s="2" t="inlineStr">
         <is>
-          <t>Independent QA. Holding MFs in the wealth ledger stays out of scope (owner Scope Exclusions); benchmark is a price index, not total return; peers limited to stored schemes</t>
+          <t>Independent QA. Holding MFs in the wealth ledger stays out of scope (owner Scope Exclusions); benchmark is a price index (the W40 Nifty 50 TR is not wired here yet); peers limited to stored schemes; tiered exit loads not modelled</t>
         </is>
       </c>
       <c r="P332" s="2" t="inlineStr">
@@ -42222,13 +42315,245 @@
       </c>
       <c r="Y332" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_mf_analytics.py | 86% of 626 lines in 3 key file(s) run by: test_auto_recover, test_w39_ml_regime_lineage_surface, test_w39_perf_budget, test_w39_ui_smoke, test_w39b_mf_analytics</t>
+          <t>tests/test_w39b_mf_analytics.py | 87% of 688 lines in 3 key file(s) run by: test_auto_recover, test_w39_mcp, test_w39_ml_regime_lineage_surface, test_w39_perf_budget, test_w39_ui_smoke, test_w39b_mf_analytics</t>
         </is>
       </c>
       <c r="Z332" s="2" t="inlineStr"/>
     </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>W39 reconciliation (owner tracker 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>W40-RISKMODEL</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>Risk &amp; Portfolio</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>Fundamental factor risk model (Barra-style)</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>Factor exposures, factor returns, covariance, specific risk and portfolio risk decomposition</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9): docs/ATIP_GAP_ANALYSIS_2026-10.md section 4 items 5 and 9; tracker next actions</t>
+        </is>
+      </c>
+      <c r="I333" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J333" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="K333" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="L333" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="M333" s="2" t="inlineStr"/>
+      <c r="N333" s="2" t="inlineStr">
+        <is>
+          <t>quant/risk_model.py: 8 styles (size, beta, momentum, residual volatility, book-to-price, earnings yield, ROE, liquidity) point in time, winsorised and cap-standardised, NSE industries (small ones pooled); daily sqrt(cap)-weighted regression with the industry constraint and robust t statistics; EWMA / Newey-West factor covariance; shrunk EWMA specific risk; decomposition of the PAPER / LIVE book (factor vs specific, per factor, marginal per stock, beta, active risk vs a cap-weighted Nifty 50 proxy); bias statistic on standard portfolios; nightly 21:45, incremental; /trading and /quant cards</t>
+        </is>
+      </c>
+      <c r="O333" s="2" t="inlineStr">
+        <is>
+          <t>Independent QA on the real database; needs filed share counts for 30+ stocks; universe and industries are today's (survivorship); no free-float data</t>
+        </is>
+      </c>
+      <c r="P333" s="2" t="inlineStr">
+        <is>
+          <t>quant/risk_model.py; portfolio/risk.py; dashboard/risk_model_routes.py</t>
+        </is>
+      </c>
+      <c r="Q333" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_risk_model.py</t>
+        </is>
+      </c>
+      <c r="R333" s="2" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S333" s="2" t="inlineStr"/>
+      <c r="T333" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="U333" s="2" t="inlineStr"/>
+      <c r="V333" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="W333" s="2" t="inlineStr">
+        <is>
+          <t>W40 developed 2026-10-09 on branch claude/wizardly-curie-fbjeoa (PR #9); independent validation PENDING</t>
+        </is>
+      </c>
+      <c r="X333" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9)</t>
+        </is>
+      </c>
+      <c r="Y333" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_risk_model.py | 76% of 1466 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model, test_w40_total_return</t>
+        </is>
+      </c>
+      <c r="Z333" s="2" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>W39 reconciliation (owner tracker 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>W40-META</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>AI/ML</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Meta-labelling of the technical signals (AFML ch. 3-4, 7, 10)</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr">
+        <is>
+          <t>A second model deciding which primary signals to take, with bet sizes</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9): docs/ATIP_GAP_ANALYSIS_2026-10.md section 4 items 5 and 9; tracker next actions</t>
+        </is>
+      </c>
+      <c r="I334" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J334" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="K334" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="L334" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="M334" s="2" t="inlineStr"/>
+      <c r="N334" s="2" t="inlineStr">
+        <is>
+          <t>ml/meta_label.py: triple-barrier labels from the signal engine's own outcome rule; 37 features known at the signal's close; sample weights by average uniqueness; purged k-fold with embargo; GBM / logistic / RF; out-of-fold precision / recall / AUC and the kept signals' expectancy vs all; AFML bet sizing (reported only); ADOPTABLE only with 200+ signals and t &gt;= 2, and the registry refuses activating anything else; Saturday retrain and 20:45 scoring, both off unless meta_label.enabled; /signals column when adopted</t>
+        </is>
+      </c>
+      <c r="O334" s="2" t="inlineStr">
+        <is>
+          <t>Owner: switch on after a few hundred closed signals exist and a version is ADOPTABLE; independent QA</t>
+        </is>
+      </c>
+      <c r="P334" s="2" t="inlineStr">
+        <is>
+          <t>ml/meta_label.py; ml/validation.py; dashboard/w40_routes.py</t>
+        </is>
+      </c>
+      <c r="Q334" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_meta_label.py</t>
+        </is>
+      </c>
+      <c r="R334" s="2" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S334" s="2" t="inlineStr"/>
+      <c r="T334" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="U334" s="2" t="inlineStr"/>
+      <c r="V334" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="W334" s="2" t="inlineStr">
+        <is>
+          <t>W40 developed 2026-10-09 on branch claude/wizardly-curie-fbjeoa (PR #9); independent validation PENDING</t>
+        </is>
+      </c>
+      <c r="X334" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9)</t>
+        </is>
+      </c>
+      <c r="Y334" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_meta_label.py | 90% of 861 lines in 3 key file(s) run by: test_auto_recover, test_w39_qa_suite, test_w39_regime_gate, test_w39_technicals, test_w40_meta_label</t>
+        </is>
+      </c>
+      <c r="Z334" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z332"/>
+  <autoFilter ref="A1:Z334"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -42239,7 +42564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z55"/>
+  <dimension ref="A1:Z57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42513,7 +42838,7 @@
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>test_paper_partial_fills_reach_the_ledger; test_entry_order_is_portable_and_numbered; test_migration_0006_numbers_old_rows_and_the_ledger_stays_append_only; test_cash_rows_and_fee_breakdown_are_validated; test_voided_transactions_are_ignored_but_kept | 77% of 317 lines in 3 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_ops_tests, test_w39_perf_budget, test_w39_performance_detail, test_wealth_api_security, test_wealth_performance (+1 more)</t>
+          <t>test_paper_partial_fills_reach_the_ledger; test_entry_order_is_portable_and_numbered; test_migration_0006_numbers_old_rows_and_the_ledger_stays_append_only; test_cash_rows_and_fee_breakdown_are_validated; test_voided_transactions_are_ignored_but_kept | 77% of 317 lines in 3 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_ops_tests, test_w39_perf_budget, test_w39_performance_detail, test_w40_total_return, test_wealth_api_security (+2 more)</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr"/>
@@ -42629,7 +42954,7 @@
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>test_model_return_is_reproducible_and_matches_a_hand_calculation; test_model_and_executable_are_reported_separately | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_model_return_is_reproducible_and_matches_a_hand_calculation; test_model_and_executable_are_reported_separately | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
@@ -42745,7 +43070,7 @@
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>test_executable_applies_slippage_costs_and_the_liquidity_cap; test_impact_slippage_uses_the_square_root_estimate_known_at_the_signal | 83% of 331 lines in 2 key file(s) run by: test_w39_backtest_partial, test_w39_contract_note_fees, test_w39_performance_detail, test_w39_untested_modules, test_wealth_performance</t>
+          <t>test_executable_applies_slippage_costs_and_the_liquidity_cap; test_impact_slippage_uses_the_square_root_estimate_known_at_the_signal | 83% of 331 lines in 2 key file(s) run by: test_w39_backtest_partial, test_w39_contract_note_fees, test_w39_performance_detail, test_w39_untested_modules, test_w40_futures_backtest, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr"/>
@@ -42861,7 +43186,7 @@
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>test_period_scope_is_separate_from_lifetime; test_xirr_and_pme_match_hand_computed_flows; test_average_cost_realized_pnl_and_fees | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_period_scope_is_separate_from_lifetime; test_xirr_and_pme_match_hand_computed_flows; test_average_cost_realized_pnl_and_fees | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr"/>
@@ -42930,22 +43255,22 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>any prices_daily symbol (NIFTY50, NIFTYBANK, midcap, smallcap, sector indices); price return over the same sessions + PME of the investor's flows; W39: days invested shown and exported</t>
+          <t>any prices_daily symbol (NIFTY50, NIFTYBANK, midcap, smallcap, sector indices); price return over the same sessions + PME of the investor's flows; W39: days invested shown and exported. W40: benchmark "nifty50tr" -- the Nifty 50 with dividends reinvested (data/total_return.py: NSE's TRI method, the price index exact, its dividend points estimated from the top 50 stored stocks by cap, picked monthly and weighted daily; nightly 21:10; GET /api/data/total-return), part of the report's audited inputs</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Total-return index (dividends) not available from the data source</t>
+          <t>Independent QA; the dividend part is an estimate (no free-float or constituent data) -- compare once with NSE's published TRI</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>wealth/perf/data.py; wealth/perf/report.py</t>
+          <t>wealth/perf/data.py; wealth/perf/report.py; data/total_return.py</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>test_benchmark_return_is_the_price_return_over_the_sessions</t>
+          <t>test_benchmark_return_is_the_price_return_over_the_sessions; tests/test_w40_total_return.py</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -42977,7 +43302,7 @@
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>test_benchmark_return_is_the_price_return_over_the_sessions | 93% of 299 lines in 2 key file(s) run by: test_w39_performance_detail, test_w39b_mf_analytics, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_benchmark_return_is_the_price_return_over_the_sessions; tests/test_w40_total_return.py | 91% of 502 lines in 3 key file(s) run by: test_w39_mcp, test_w39_performance_detail, test_w39b_mf_analytics, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr"/>
@@ -43093,7 +43418,7 @@
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>test_costs_reconcile_with_dividend_tax_fee_rows_and_a_capped_sell; test_statutory_estimate_itemises_paper_brokerage_only_trades; tests/test_w39_contract_note_fees.py | 89% of 587 lines in 2 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_costs_reconcile_with_dividend_tax_fee_rows_and_a_capped_sell; test_statutory_estimate_itemises_paper_brokerage_only_trades; tests/test_w39_contract_note_fees.py | 89% of 587 lines in 2 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr"/>
@@ -43209,7 +43534,7 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win; test_position_attribution_identity | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win; test_position_attribution_identity | 88% of 230 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr"/>
@@ -43325,7 +43650,7 @@
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>test_risk_metrics_match_independent_formulas; test_cagr_annualises_a_full_year; test_xirr_one_year_ten_percent; test_trade_stats | 96% of 216 lines in 2 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_cpcv_pbo, test_w39b_mf_analytics, test_wealth_math (+1 more)</t>
+          <t>test_risk_metrics_match_independent_formulas; test_cagr_annualises_a_full_year; test_xirr_one_year_ten_percent; test_trade_stats | 96% of 217 lines in 2 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39_mcp, test_w39_performance_detail, test_w39_qa_suite, test_w39_untested_modules, test_w39b_bayes_optimize, test_w39b_cpcv_dominance (+7 more)</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr"/>
@@ -43441,7 +43766,7 @@
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win | 92% of 461 lines in 2 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_sizing_effect_completes_the_decomposition_and_exact_links_win | 92% of 461 lines in 2 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr"/>
@@ -43557,7 +43882,7 @@
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>test_risk_contribution_reconciles_and_groups_sum_to_the_total; test_contributions_reconcile_to_the_total | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_wealth_performance</t>
+          <t>test_risk_contribution_reconciles_and_groups_sum_to_the_total; test_contributions_reconcile_to_the_total | 94% of 371 lines in 1 key file(s) run by: test_w39_contract_note_fees, test_w39_performance_detail, test_w40_total_return, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr"/>
@@ -43789,7 +44114,7 @@
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>test_verify_reproduces_and_detects_changed_inputs | 95% of 231 lines in 1 key file(s) run by: test_w39_performance_detail, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_verify_reproduces_and_detects_changed_inputs | 96% of 231 lines in 1 key file(s) run by: test_w39_performance_detail, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr"/>
@@ -43905,7 +44230,7 @@
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>test_export_carries_every_section_with_the_reports_numbers; test_strategy_filter_limits_the_actual_portfolio; test_printable_html_has_the_csv_sections_and_numbers_and_escapes_text | 87% of 594 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_performance_detail, test_w39_ui_smoke, test_wealth_api_security, test_wealth_performance</t>
+          <t>test_export_carries_every_section_with_the_reports_numbers; test_strategy_filter_limits_the_actual_portfolio; test_printable_html_has_the_csv_sections_and_numbers_and_escapes_text | 87% of 594 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_performance_detail, test_w39_ui_smoke, test_w40_total_return, test_wealth_api_security, test_wealth_performance</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr"/>
@@ -44021,7 +44346,7 @@
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>test_a_trade_on_a_market_holiday_counts_on_the_next_session; test_missing_bars_are_reported_not_hidden; test_a_bonus_issue_keeps_value_and_cost; test_an_opening_position_is_measured_from_that_days_close; test_split_between_buy_and_today_moves_neither_value_nor_return | 89% of 1179 lines in 6 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_notify_transactions, test_w39_performance_detail, test_w39b_mf_analytics, test_wealth_api_security, test_wealth_math, test_wealth_performance (+1 more)</t>
+          <t>test_a_trade_on_a_market_holiday_counts_on_the_next_session; test_missing_bars_are_reported_not_hidden; test_a_bonus_issue_keeps_value_and_cost; test_an_opening_position_is_measured_from_that_days_close; test_split_between_buy_and_today_moves_neither_value_nor_return | 90% of 1207 lines in 6 key file(s) run by: test_w37_brokers_multi_asset, test_w39_contract_note_fees, test_w39_mcp, test_w39_notify_transactions, test_w39_performance_detail, test_w39b_mf_analytics, test_w40_total_return, test_wealth_api_security (+3 more)</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr"/>
@@ -44253,7 +44578,7 @@
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_history.py; tests/test_w39b_merge.py | 51% of 1001 lines in 3 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_ops_tests (+3 more)</t>
+          <t>tests/test_w39_history.py; tests/test_w39b_merge.py | 50% of 1001 lines in 3 key file(s) run by: test_corporate_actions, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w39_history, test_w39_notify_transactions, test_w39_ops_tests (+3 more)</t>
         </is>
       </c>
       <c r="Z17" s="2" t="inlineStr"/>
@@ -44322,7 +44647,7 @@
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>W26 stock panel + W39: 3Y / 5Y / All, daily / weekly / monthly bars, SMA 20/50/200, EMA 21, Bollinger, log scale, multi-year returns; checked in headless Chromium</t>
+          <t>W26 stock panel + W39: 3Y / 5Y / All, daily / weekly / monthly bars, SMA 20/50/200, EMA 21, Bollinger, log scale, multi-year returns; checked in headless Chromium. W39b: signal / pattern marks. W40: RSI 14 and MACD 12-26-9 panels (the server's definitions), an intraday chart (1D / 5D on 15-minute bars, session VWAP, previous close, intraday scan marks; GET /api/stock/{symbol}/intraday) and the on-demand 75-minute rating</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -44337,7 +44662,7 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>test_stock_history_reports_multi_year_returns</t>
+          <t>test_stock_history_reports_multi_year_returns; tests/test_w40_stock_chart.py</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
@@ -44369,7 +44694,7 @@
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>test_stock_history_reports_multi_year_returns | 84% of 113 lines in 1 key file(s) run by: test_auto_recover, test_w39_owner_notes, test_w39_perf_budget, test_w39b_patterns_more</t>
+          <t>test_stock_history_reports_multi_year_returns; tests/test_w40_stock_chart.py | 88% of 248 lines in 1 key file(s) run by: test_auto_recover, test_w39_mcp, test_w39_owner_notes, test_w39_perf_budget, test_w39b_patterns_more, test_w39b_tf75_signals, test_w40_stock_chart</t>
         </is>
       </c>
       <c r="Z18" s="2" t="inlineStr"/>
@@ -44485,7 +44810,7 @@
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_risk_gateway.py | 51% of 1617 lines in 3 key file(s) run by: test_auto_recover, test_corporate_actions, test_job_monitoring, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w38_platform_compliance (+10 more)</t>
+          <t>tests/test_w39_risk_gateway.py | 51% of 1622 lines in 3 key file(s) run by: test_auto_recover, test_corporate_actions, test_job_monitoring, test_regressions, test_risk_controls, test_signal_pipeline, test_strategy_live, test_w38_platform_compliance (+15 more)</t>
         </is>
       </c>
       <c r="Z19" s="2" t="inlineStr"/>
@@ -44601,7 +44926,7 @@
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_quant_portfolio.py | 61% of 266 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio</t>
+          <t>tests/test_w39_quant_portfolio.py | 68% of 269 lines in 1 key file(s) run by: test_auto_recover, test_w36_ml_strategy_tooling, test_w39_api_contract, test_w39_quant_portfolio, test_w40_risk_model</t>
         </is>
       </c>
       <c r="Z20" s="2" t="inlineStr"/>
@@ -44949,7 +45274,7 @@
       </c>
       <c r="Y23" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_ml_regime_lineage_surface.py | 86% of 140 lines in 1 key file(s) run by: test_w36_ml_strategy_tooling, test_w39_ml_regime_lineage_surface, test_w39_options</t>
+          <t>tests/test_w39_ml_regime_lineage_surface.py | 86% of 140 lines in 1 key file(s) run by: test_w36_ml_strategy_tooling, test_w39_ml_regime_lineage_surface, test_w39_options, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z23" s="2" t="inlineStr"/>
@@ -45065,7 +45390,7 @@
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_ml_regime_lineage_surface.py | 87% of 341 lines in 2 key file(s) run by: test_w39_ml_regime_lineage_surface</t>
+          <t>tests/test_w39_ml_regime_lineage_surface.py | 87% of 341 lines in 2 key file(s) run by: test_w39_ml_regime_lineage_surface, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z24" s="2" t="inlineStr"/>
@@ -45181,7 +45506,7 @@
       </c>
       <c r="Y25" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_ml_regime_lineage_surface.py | 73% of 148 lines in 1 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite</t>
+          <t>tests/test_w39_ml_regime_lineage_surface.py | 88% of 154 lines in 1 key file(s) run by: test_auto_recover, test_w39_api_contract, test_w39_ml_regime_lineage_surface, test_w39_qa_suite, test_w40_meta_label</t>
         </is>
       </c>
       <c r="Z25" s="2" t="inlineStr"/>
@@ -45297,7 +45622,7 @@
       </c>
       <c r="Y26" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_backtest.py | 82% of 126 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39b_cpcv_pbo</t>
+          <t>tests/test_w39_backtest.py | 83% of 126 lines in 1 key file(s) run by: test_w39_backtest, test_w39_backtest_partial, test_w39b_bayes_optimize, test_w39b_cpcv_dominance, test_w39b_cpcv_pbo, test_w39b_event_driven_skips, test_w40_futures_backtest</t>
         </is>
       </c>
       <c r="Z26" s="2" t="inlineStr"/>
@@ -46337,7 +46662,7 @@
       </c>
       <c r="Y35" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_options.py | 88% of 209 lines in 1 key file(s) run by: test_w39_options</t>
+          <t>tests/test_w39_options.py | 88% of 209 lines in 1 key file(s) run by: test_signal_pipeline, test_w39_options, test_w40_option_intents</t>
         </is>
       </c>
       <c r="Z35" s="2" t="inlineStr"/>
@@ -46453,7 +46778,7 @@
       </c>
       <c r="Y36" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_technicals.py | 88% of 820 lines in 2 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+9 more)</t>
+          <t>tests/test_w39_technicals.py | 89% of 885 lines in 2 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+12 more)</t>
         </is>
       </c>
       <c r="Z36" s="2" t="inlineStr"/>
@@ -46685,7 +47010,7 @@
       </c>
       <c r="Y38" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_regime_gate.py | 83% of 248 lines in 1 key file(s) run by: test_w39_delivery, test_w39_event_calendar, test_w39_market_pulse, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_regime_gate.py | 83% of 248 lines in 1 key file(s) run by: test_w39_delivery, test_w39_event_calendar, test_w39_market_pulse, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_technicals (+6 more)</t>
         </is>
       </c>
       <c r="Z38" s="2" t="inlineStr"/>
@@ -46801,7 +47126,7 @@
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_track_record.py | 84% of 522 lines in 1 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+6 more)</t>
+          <t>tests/test_w39_track_record.py | 85% of 587 lines in 1 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+9 more)</t>
         </is>
       </c>
       <c r="Z39" s="2" t="inlineStr"/>
@@ -46917,7 +47242,7 @@
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_weekly.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_weekly.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z40" s="2" t="inlineStr"/>
@@ -47033,7 +47358,7 @@
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_patterns.py; tests/test_w39b_patterns_more.py | 93% of 491 lines in 2 key file(s) run by: test_auto_recover, test_w39_delivery, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_patterns.py; tests/test_w39b_patterns_more.py | 93% of 626 lines in 2 key file(s) run by: test_auto_recover, test_w39_delivery, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr"/>
@@ -47149,7 +47474,7 @@
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_rs_line.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_rs_line.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z42" s="2" t="inlineStr"/>
@@ -47265,7 +47590,7 @@
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_delivery.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals (+4 more)</t>
+          <t>tests/test_w39_delivery.py | 95% of 298 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+7 more)</t>
         </is>
       </c>
       <c r="Z43" s="2" t="inlineStr"/>
@@ -47613,7 +47938,7 @@
       </c>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_intraday.py | 88% of 225 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals, test_w39_weekly, test_w39b_tf75</t>
+          <t>tests/test_w39_intraday.py | 88% of 225 lines in 1 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_regime_gate, test_w39_rs_line, test_w39_technicals, test_w39_weekly, test_w39b_tf75 (+2 more)</t>
         </is>
       </c>
       <c r="Z46" s="2" t="inlineStr"/>
@@ -48030,7 +48355,7 @@
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>tools/atip_mcp.py</t>
+          <t>tools/atip_mcp.py; W40: 20 tools -- adds dvm, earnings_surprise, mf_search / mf_analytics / mf_sip / mf_compare, backtest_validation (stored CPCV / PBO) and chart_marks, each checked under query_only</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
@@ -48077,7 +48402,7 @@
       </c>
       <c r="Y50" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39_mcp.py | 83% of 184 lines in 1 key file(s) run by: test_w39_mcp</t>
+          <t>tests/test_w39_mcp.py | 91% of 331 lines in 1 key file(s) run by: test_w39_mcp</t>
         </is>
       </c>
       <c r="Z50" s="2" t="inlineStr"/>
@@ -48267,7 +48592,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>Independent QA; no live intraday refresh (once a day, as of the close); /signals has no 75-minute column</t>
+          <t>Independent QA. W40: a 75m column on /signals and GET /api/stock/{symbol}/rating-75 (on demand from the stored 15-minute bars, completed bars only); the /signals column is still the 20:30 snapshot</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -48277,7 +48602,7 @@
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_tf75.py</t>
+          <t>tests/test_w39b_tf75.py; tests/test_w39b_tf75_signals.py</t>
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr">
@@ -48309,7 +48634,7 @@
       </c>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_tf75.py | 88% of 1266 lines in 3 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+10 more)</t>
+          <t>tests/test_w39b_tf75.py; tests/test_w39b_tf75_signals.py | 89% of 1331 lines in 3 key file(s) run by: test_w39_delivery, test_w39_intraday, test_w39_mcp, test_w39_owner_notes, test_w39_patterns, test_w39_perf_budget, test_w39_regime_gate, test_w39_rs_line (+13 more)</t>
         </is>
       </c>
       <c r="Z52" s="2" t="inlineStr"/>
@@ -48425,7 +48750,7 @@
       </c>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_dvm.py | 86% of 1041 lines in 3 key file(s) run by: test_auto_recover, test_w39_depth20, test_w39_event_calendar, test_w39_global_sync, test_w39_intraday, test_w39_market_pulse, test_w39_mcp, test_w39_options (+12 more)</t>
+          <t>tests/test_w39b_dvm.py | 86% of 1044 lines in 3 key file(s) run by: test_auto_recover, test_w39_depth20, test_w39_event_calendar, test_w39_global_sync, test_w39_intraday, test_w39_market_pulse, test_w39_mcp, test_w39_options (+14 more)</t>
         </is>
       </c>
       <c r="Z53" s="2" t="inlineStr"/>
@@ -48541,7 +48866,7 @@
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_earnings_surprise.py | 85% of 905 lines in 2 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+6 more)</t>
+          <t>tests/test_w39b_earnings_surprise.py | 86% of 970 lines in 2 key file(s) run by: test_w39_delivery, test_w39_mcp, test_w39_patterns, test_w39_regime_gate, test_w39_rs_line, test_w39_scorecard, test_w39_screener, test_w39_technicals (+9 more)</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
@@ -48614,12 +48939,12 @@
       <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>data/mf_analytics.py: point-to-point and CAGR returns, 1Y / 3Y rolling returns with hurdle stats, volatility / Sharpe / Sortino, drawdown with dates, beta / alpha / tracking error vs a price index, SIP and lump-sum XIRR, category rank among stored schemes, side-by-side compare; 3 read-only GET routes; scheme detail card on /data-platform</t>
+          <t>data/mf_analytics.py: point-to-point and CAGR returns, 1Y / 3Y rolling returns with hurdle stats, volatility / Sharpe / Sortino, drawdown with dates, beta / alpha / tracking error vs a price index, SIP and lump-sum XIRR, category rank among stored schemes, side-by-side compare; 3 read-only GET routes; scheme detail card on /data-platform. W40: step-up SIP, stamp duty (0.005 %) and units rounded down to 3 decimals by default, optional flat exit load per instalment; volatility annualised by the NAVs actually observed a year (not a fixed 252)</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>Independent QA. Holding MFs in the wealth ledger stays out of scope (owner Scope Exclusions); benchmark is a price index, not total return; peers limited to stored schemes</t>
+          <t>Independent QA. Holding MFs in the wealth ledger stays out of scope (owner Scope Exclusions); benchmark is a price index (the W40 Nifty 50 TR is not wired here yet); peers limited to stored schemes; tiered exit loads not modelled</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -48661,13 +48986,245 @@
       </c>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>tests/test_w39b_mf_analytics.py | 86% of 626 lines in 3 key file(s) run by: test_auto_recover, test_w39_ml_regime_lineage_surface, test_w39_perf_budget, test_w39_ui_smoke, test_w39b_mf_analytics</t>
+          <t>tests/test_w39b_mf_analytics.py | 87% of 688 lines in 3 key file(s) run by: test_auto_recover, test_w39_mcp, test_w39_ml_regime_lineage_surface, test_w39_perf_budget, test_w39_ui_smoke, test_w39b_mf_analytics</t>
         </is>
       </c>
       <c r="Z55" s="2" t="inlineStr"/>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>W39 reconciliation (owner tracker 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>W40-RISKMODEL</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Risk &amp; Portfolio</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Fundamental factor risk model (Barra-style)</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Factor exposures, factor returns, covariance, specific risk and portfolio risk decomposition</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9): docs/ATIP_GAP_ANALYSIS_2026-10.md section 4 items 5 and 9; tracker next actions</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J56" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="K56" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>quant/risk_model.py: 8 styles (size, beta, momentum, residual volatility, book-to-price, earnings yield, ROE, liquidity) point in time, winsorised and cap-standardised, NSE industries (small ones pooled); daily sqrt(cap)-weighted regression with the industry constraint and robust t statistics; EWMA / Newey-West factor covariance; shrunk EWMA specific risk; decomposition of the PAPER / LIVE book (factor vs specific, per factor, marginal per stock, beta, active risk vs a cap-weighted Nifty 50 proxy); bias statistic on standard portfolios; nightly 21:45, incremental; /trading and /quant cards</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Independent QA on the real database; needs filed share counts for 30+ stocks; universe and industries are today's (survivorship); no free-float data</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>quant/risk_model.py; portfolio/risk.py; dashboard/risk_model_routes.py</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_risk_model.py</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr"/>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>W40 developed 2026-10-09 on branch claude/wizardly-curie-fbjeoa (PR #9); independent validation PENDING</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9)</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_risk_model.py | 76% of 1466 lines in 3 key file(s) run by: test_auto_recover, test_w39_perf_budget, test_w39_qa_suite, test_w39_quant_portfolio, test_w39_ui_smoke, test_w40_risk_model, test_w40_total_return</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>W39 reconciliation (owner tracker 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>W40-META</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>AI/ML</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Meta-labelling of the technical signals (AFML ch. 3-4, 7, 10)</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>A second model deciding which primary signals to take, with bet sizes</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9): docs/ATIP_GAP_ANALYSIS_2026-10.md section 4 items 5 and 9; tracker next actions</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J57" s="18" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED BUT NOT VERIFIED</t>
+        </is>
+      </c>
+      <c r="K57" s="14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>ml/meta_label.py: triple-barrier labels from the signal engine's own outcome rule; 37 features known at the signal's close; sample weights by average uniqueness; purged k-fold with embargo; GBM / logistic / RF; out-of-fold precision / recall / AUC and the kept signals' expectancy vs all; AFML bet sizing (reported only); ADOPTABLE only with 200+ signals and t &gt;= 2, and the registry refuses activating anything else; Saturday retrain and 20:45 scoring, both off unless meta_label.enabled; /signals column when adopted</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Owner: switch on after a few hundred closed signals exist and a version is ADOPTABLE; independent QA</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>ml/meta_label.py; ml/validation.py; dashboard/w40_routes.py</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_meta_label.py</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Claude (development)</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr"/>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="U57" s="2" t="inlineStr"/>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>W40 developed 2026-10-09 on branch claude/wizardly-curie-fbjeoa (PR #9); independent validation PENDING</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>W40 (PR #9)</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_w40_meta_label.py | 90% of 861 lines in 3 key file(s) run by: test_auto_recover, test_w39_qa_suite, test_w39_regime_gate, test_w39_technicals, test_w40_meta_label</t>
+        </is>
+      </c>
+      <c r="Z57" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z55"/>
+  <autoFilter ref="A1:Z57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -49352,7 +49909,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>[2026-10-07] 49/49 features developed (14 COMPLETED, 35 awaiting independent QA); automated tests: 35 covered, 14 partly, 0 none</t>
+          <t>[2026-10-07] 49/49 features developed (14 COMPLETED, 35 awaiting independent QA); automated tests: 36 covered, 13 partly, 0 none</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -49392,7 +49949,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>[2026-10-07] 18/19 features developed (16 COMPLETED, 2 awaiting independent QA); automated tests: 9 covered, 9 partly, 0 none; BLOCKED: SE-05</t>
+          <t>[2026-10-07] 18/19 features developed (16 COMPLETED, 2 awaiting independent QA); automated tests: 11 covered, 7 partly, 0 none; BLOCKED: SE-05</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -49432,7 +49989,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>[2026-10-07] 32/32 features developed (15 COMPLETED, 17 awaiting independent QA); automated tests: 19 covered, 13 partly, 0 none</t>
+          <t>[2026-10-07] 32/32 features developed (15 COMPLETED, 17 awaiting independent QA); automated tests: 22 covered, 10 partly, 0 none</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -50160,7 +50717,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>[2026-10-07] 10/10 features developed (0 COMPLETED, 10 awaiting independent QA); automated tests: 5 covered, 5 partly, 0 none</t>
+          <t>[2026-10-07] 10/10 features developed (0 COMPLETED, 10 awaiting independent QA); automated tests: 6 covered, 4 partly, 0 none</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -50454,7 +51011,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>[2026-10-07] 6/6 features developed (0 COMPLETED, 6 awaiting independent QA); automated tests: 1 covered, 5 partly, 0 none</t>
+          <t>[2026-10-07] 6/6 features developed (0 COMPLETED, 6 awaiting independent QA); automated tests: 3 covered, 3 partly, 0 none</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -50832,7 +51389,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>[2026-10-07] 57/59 features developed (1 COMPLETED, 56 awaiting independent QA); automated tests: 58 covered, 0 partly, 0 none; BLOCKED: EX-19; open: QA-001</t>
+          <t>[2026-10-07] 59/61 features developed (1 COMPLETED, 58 awaiting independent QA); automated tests: 60 covered, 0 partly, 0 none; BLOCKED: EX-19; open: QA-001</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -50990,7 +51547,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>79.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="G4" t="n">
         <v>41</v>
@@ -51022,7 +51579,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>85</v>
+        <v>85.5</v>
       </c>
       <c r="G5" t="n">
         <v>19</v>
@@ -52203,17 +52760,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>any prices_daily symbol (NIFTY50, NIFTYBANK, midcap, smallcap, sector indices); price return over the same sessions + PME of the investor's flows; W39: days invested shown and exported</t>
+          <t>any prices_daily symbol (NIFTY50, NIFTYBANK, midcap, smallcap, sector indices); price return over the same sessions + PME of the investor's flows; W39: days invested shown and exported. W40: benchmark "nifty50tr" -- the Nifty 50 with dividends reinvested (data/total_return.py: NSE's TRI method, the price index exact, its dividend points estimated from the top 50 stored stocks by cap, picked monthly and weighted daily; nightly 21:10; GET /api/data/total-return), part of the report's audited inputs</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>test_benchmark_return_is_the_price_return_over_the_sessions</t>
+          <t>test_benchmark_return_is_the_price_return_over_the_sessions; tests/test_w40_total_return.py</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Total-return index (dividends) not available from the data source</t>
+          <t>Independent QA; the dividend part is an estimate (no free-float or constituent data) -- compare once with NSE's published TRI</t>
         </is>
       </c>
     </row>

</xml_diff>